<commit_message>
fix(orcamento): planejado dos CLT volta ao valor orcado na ficha
A divisao em salario bruto + encargos colocava R$ 2.886,91 como
planejado da Geovanna (e R$ 2.570,52 do Vinicius). Esses valores sao o
salario que eles recebem hoje, nao o que foi orcado — a ficha orcou
R$ 4.825,52 e R$ 5.416,52 de custo total, e planejado tem que ser o
que foi orcado.

Cada um volta a uma linha unica com o valor da ficha. O bruto conhecido
fica registrado na descricao, e o realizado das duas linhas fica em
branco ate vir o custo total: lancar so o bruto contra um orcado de
custo total mostraria economia inexistente de R$ 1.938,61/mes na
Geovanna e R$ 2.846,01/mes no Vinicius.

Totais preservados: Juridico R$ 290.730,42, TI R$ 256.818,30, geral
R$ 547.548,72. O plano de contas "Encargos e Beneficios - CLT" deixa de
existir.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_JURIDICO_2026.xlsx
+++ b/orcamento/Orcamento_JURIDICO_2026.xlsx
@@ -17,8 +17,8 @@
     <sheet name="Como usar" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Comparativo'!$A$5:$N$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Planejado'!$A$4:$T$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Comparativo'!$A$5:$N$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Planejado'!$A$4:$T$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1115,15 +1115,15 @@
         </is>
       </c>
       <c r="C6" s="8">
-        <f>SUMIFS(Planejado!$T$5:$T$14,Planejado!$B$5:$B$14,"Jurídico",Planejado!$C$5:$C$14,"Equipe")</f>
+        <f>SUMIFS(Planejado!$T$5:$T$13,Planejado!$B$5:$B$13,"Jurídico",Planejado!$C$5:$C$13,"Equipe")</f>
         <v/>
       </c>
       <c r="D6" s="8">
-        <f>SUMIFS(Comparativo!$I$6:$I$15,Comparativo!$B$6:$B$15,"Jurídico",Comparativo!$C$6:$C$15,"Equipe")</f>
+        <f>SUMIFS(Comparativo!$I$6:$I$14,Comparativo!$B$6:$B$14,"Jurídico",Comparativo!$C$6:$C$14,"Equipe")</f>
         <v/>
       </c>
       <c r="E6" s="8">
-        <f>SUMIFS(Comparativo!$J$6:$J$15,Comparativo!$B$6:$B$15,"Jurídico",Comparativo!$C$6:$C$15,"Equipe")</f>
+        <f>SUMIFS(Comparativo!$J$6:$J$14,Comparativo!$B$6:$B$14,"Jurídico",Comparativo!$C$6:$C$14,"Equipe")</f>
         <v/>
       </c>
       <c r="F6" s="8">
@@ -1139,7 +1139,7 @@
         <v/>
       </c>
       <c r="I6" s="10">
-        <f>COUNTIFS(Comparativo!$P$6:$P$15,"&gt;0",Comparativo!$B$6:$B$15,"Jurídico",Comparativo!$C$6:$C$15,"Equipe")&amp;" de "&amp;COUNTIFS(Comparativo!$A$6:$A$15,"?*",Comparativo!$B$6:$B$15,"Jurídico",Comparativo!$C$6:$C$15,"Equipe")</f>
+        <f>COUNTIFS(Comparativo!$P$6:$P$14,"&gt;0",Comparativo!$B$6:$B$14,"Jurídico",Comparativo!$C$6:$C$14,"Equipe")&amp;" de "&amp;COUNTIFS(Comparativo!$A$6:$A$14,"?*",Comparativo!$B$6:$B$14,"Jurídico",Comparativo!$C$6:$C$14,"Equipe")</f>
         <v/>
       </c>
     </row>
@@ -1155,15 +1155,15 @@
         </is>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Planejado!$T$5:$T$14,Planejado!$B$5:$B$14,"Jurídico",Planejado!$C$5:$C$14,"Despesas")</f>
+        <f>SUMIFS(Planejado!$T$5:$T$13,Planejado!$B$5:$B$13,"Jurídico",Planejado!$C$5:$C$13,"Despesas")</f>
         <v/>
       </c>
       <c r="D7" s="8">
-        <f>SUMIFS(Comparativo!$I$6:$I$15,Comparativo!$B$6:$B$15,"Jurídico",Comparativo!$C$6:$C$15,"Despesas")</f>
+        <f>SUMIFS(Comparativo!$I$6:$I$14,Comparativo!$B$6:$B$14,"Jurídico",Comparativo!$C$6:$C$14,"Despesas")</f>
         <v/>
       </c>
       <c r="E7" s="8">
-        <f>SUMIFS(Comparativo!$J$6:$J$15,Comparativo!$B$6:$B$15,"Jurídico",Comparativo!$C$6:$C$15,"Despesas")</f>
+        <f>SUMIFS(Comparativo!$J$6:$J$14,Comparativo!$B$6:$B$14,"Jurídico",Comparativo!$C$6:$C$14,"Despesas")</f>
         <v/>
       </c>
       <c r="F7" s="8">
@@ -1179,7 +1179,7 @@
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>COUNTIFS(Comparativo!$P$6:$P$15,"&gt;0",Comparativo!$B$6:$B$15,"Jurídico",Comparativo!$C$6:$C$15,"Despesas")&amp;" de "&amp;COUNTIFS(Comparativo!$A$6:$A$15,"?*",Comparativo!$B$6:$B$15,"Jurídico",Comparativo!$C$6:$C$15,"Despesas")</f>
+        <f>COUNTIFS(Comparativo!$P$6:$P$14,"&gt;0",Comparativo!$B$6:$B$14,"Jurídico",Comparativo!$C$6:$C$14,"Despesas")&amp;" de "&amp;COUNTIFS(Comparativo!$A$6:$A$14,"?*",Comparativo!$B$6:$B$14,"Jurídico",Comparativo!$C$6:$C$14,"Despesas")</f>
         <v/>
       </c>
     </row>
@@ -1195,15 +1195,15 @@
         </is>
       </c>
       <c r="C8" s="12">
-        <f>SUMIFS(Planejado!$T$5:$T$14,Planejado!$B$5:$B$14,"Jurídico")</f>
+        <f>SUMIFS(Planejado!$T$5:$T$13,Planejado!$B$5:$B$13,"Jurídico")</f>
         <v/>
       </c>
       <c r="D8" s="12">
-        <f>SUMIFS(Comparativo!$I$6:$I$15,Comparativo!$B$6:$B$15,"Jurídico")</f>
+        <f>SUMIFS(Comparativo!$I$6:$I$14,Comparativo!$B$6:$B$14,"Jurídico")</f>
         <v/>
       </c>
       <c r="E8" s="12">
-        <f>SUMIFS(Comparativo!$J$6:$J$15,Comparativo!$B$6:$B$15,"Jurídico")</f>
+        <f>SUMIFS(Comparativo!$J$6:$J$14,Comparativo!$B$6:$B$14,"Jurídico")</f>
         <v/>
       </c>
       <c r="F8" s="12">
@@ -1219,7 +1219,7 @@
         <v/>
       </c>
       <c r="I8" s="14">
-        <f>COUNTIFS(Comparativo!$P$6:$P$15,"&gt;0",Comparativo!$B$6:$B$15,"Jurídico")&amp;" de "&amp;COUNTIFS(Comparativo!$A$6:$A$15,"?*",Comparativo!$B$6:$B$15,"Jurídico")</f>
+        <f>COUNTIFS(Comparativo!$P$6:$P$14,"&gt;0",Comparativo!$B$6:$B$14,"Jurídico")&amp;" de "&amp;COUNTIFS(Comparativo!$A$6:$A$14,"?*",Comparativo!$B$6:$B$14,"Jurídico")</f>
         <v/>
       </c>
     </row>
@@ -1273,23 +1273,23 @@
         <v>1</v>
       </c>
       <c r="B13" s="17">
-        <f>IFERROR(INDEX(Comparativo!$D$6:$D$15,MATCH(LARGE(Comparativo!$O$6:$O$15,A13),Comparativo!$O$6:$O$15,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$D$6:$D$14,MATCH(LARGE(Comparativo!$O$6:$O$14,A13),Comparativo!$O$6:$O$14,0)),"")</f>
         <v/>
       </c>
       <c r="C13" s="17">
-        <f>IFERROR(INDEX(Comparativo!$B$6:$B$15,MATCH(LARGE(Comparativo!$O$6:$O$15,A13),Comparativo!$O$6:$O$15,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$B$6:$B$14,MATCH(LARGE(Comparativo!$O$6:$O$14,A13),Comparativo!$O$6:$O$14,0)),"")</f>
         <v/>
       </c>
       <c r="D13" s="18">
-        <f>IFERROR(INDEX(Comparativo!$I$6:$I$15,MATCH(LARGE(Comparativo!$O$6:$O$15,A13),Comparativo!$O$6:$O$15,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$I$6:$I$14,MATCH(LARGE(Comparativo!$O$6:$O$14,A13),Comparativo!$O$6:$O$14,0)),"")</f>
         <v/>
       </c>
       <c r="E13" s="18">
-        <f>IFERROR(INDEX(Comparativo!$J$6:$J$15,MATCH(LARGE(Comparativo!$O$6:$O$15,A13),Comparativo!$O$6:$O$15,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$J$6:$J$14,MATCH(LARGE(Comparativo!$O$6:$O$14,A13),Comparativo!$O$6:$O$14,0)),"")</f>
         <v/>
       </c>
       <c r="F13" s="18">
-        <f>IFERROR(INDEX(Comparativo!$K$6:$K$15,MATCH(LARGE(Comparativo!$O$6:$O$15,A13),Comparativo!$O$6:$O$15,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$K$6:$K$14,MATCH(LARGE(Comparativo!$O$6:$O$14,A13),Comparativo!$O$6:$O$14,0)),"")</f>
         <v/>
       </c>
       <c r="G13" s="19">
@@ -1302,23 +1302,23 @@
         <v>2</v>
       </c>
       <c r="B14" s="17">
-        <f>IFERROR(INDEX(Comparativo!$D$6:$D$15,MATCH(LARGE(Comparativo!$O$6:$O$15,A14),Comparativo!$O$6:$O$15,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$D$6:$D$14,MATCH(LARGE(Comparativo!$O$6:$O$14,A14),Comparativo!$O$6:$O$14,0)),"")</f>
         <v/>
       </c>
       <c r="C14" s="17">
-        <f>IFERROR(INDEX(Comparativo!$B$6:$B$15,MATCH(LARGE(Comparativo!$O$6:$O$15,A14),Comparativo!$O$6:$O$15,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$B$6:$B$14,MATCH(LARGE(Comparativo!$O$6:$O$14,A14),Comparativo!$O$6:$O$14,0)),"")</f>
         <v/>
       </c>
       <c r="D14" s="18">
-        <f>IFERROR(INDEX(Comparativo!$I$6:$I$15,MATCH(LARGE(Comparativo!$O$6:$O$15,A14),Comparativo!$O$6:$O$15,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$I$6:$I$14,MATCH(LARGE(Comparativo!$O$6:$O$14,A14),Comparativo!$O$6:$O$14,0)),"")</f>
         <v/>
       </c>
       <c r="E14" s="18">
-        <f>IFERROR(INDEX(Comparativo!$J$6:$J$15,MATCH(LARGE(Comparativo!$O$6:$O$15,A14),Comparativo!$O$6:$O$15,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$J$6:$J$14,MATCH(LARGE(Comparativo!$O$6:$O$14,A14),Comparativo!$O$6:$O$14,0)),"")</f>
         <v/>
       </c>
       <c r="F14" s="18">
-        <f>IFERROR(INDEX(Comparativo!$K$6:$K$15,MATCH(LARGE(Comparativo!$O$6:$O$15,A14),Comparativo!$O$6:$O$15,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$K$6:$K$14,MATCH(LARGE(Comparativo!$O$6:$O$14,A14),Comparativo!$O$6:$O$14,0)),"")</f>
         <v/>
       </c>
       <c r="G14" s="19">
@@ -1331,23 +1331,23 @@
         <v>3</v>
       </c>
       <c r="B15" s="17">
-        <f>IFERROR(INDEX(Comparativo!$D$6:$D$15,MATCH(LARGE(Comparativo!$O$6:$O$15,A15),Comparativo!$O$6:$O$15,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$D$6:$D$14,MATCH(LARGE(Comparativo!$O$6:$O$14,A15),Comparativo!$O$6:$O$14,0)),"")</f>
         <v/>
       </c>
       <c r="C15" s="17">
-        <f>IFERROR(INDEX(Comparativo!$B$6:$B$15,MATCH(LARGE(Comparativo!$O$6:$O$15,A15),Comparativo!$O$6:$O$15,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$B$6:$B$14,MATCH(LARGE(Comparativo!$O$6:$O$14,A15),Comparativo!$O$6:$O$14,0)),"")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>IFERROR(INDEX(Comparativo!$I$6:$I$15,MATCH(LARGE(Comparativo!$O$6:$O$15,A15),Comparativo!$O$6:$O$15,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$I$6:$I$14,MATCH(LARGE(Comparativo!$O$6:$O$14,A15),Comparativo!$O$6:$O$14,0)),"")</f>
         <v/>
       </c>
       <c r="E15" s="18">
-        <f>IFERROR(INDEX(Comparativo!$J$6:$J$15,MATCH(LARGE(Comparativo!$O$6:$O$15,A15),Comparativo!$O$6:$O$15,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$J$6:$J$14,MATCH(LARGE(Comparativo!$O$6:$O$14,A15),Comparativo!$O$6:$O$14,0)),"")</f>
         <v/>
       </c>
       <c r="F15" s="18">
-        <f>IFERROR(INDEX(Comparativo!$K$6:$K$15,MATCH(LARGE(Comparativo!$O$6:$O$15,A15),Comparativo!$O$6:$O$15,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$K$6:$K$14,MATCH(LARGE(Comparativo!$O$6:$O$14,A15),Comparativo!$O$6:$O$14,0)),"")</f>
         <v/>
       </c>
       <c r="G15" s="19">
@@ -1360,23 +1360,23 @@
         <v>4</v>
       </c>
       <c r="B16" s="17">
-        <f>IFERROR(INDEX(Comparativo!$D$6:$D$15,MATCH(LARGE(Comparativo!$O$6:$O$15,A16),Comparativo!$O$6:$O$15,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$D$6:$D$14,MATCH(LARGE(Comparativo!$O$6:$O$14,A16),Comparativo!$O$6:$O$14,0)),"")</f>
         <v/>
       </c>
       <c r="C16" s="17">
-        <f>IFERROR(INDEX(Comparativo!$B$6:$B$15,MATCH(LARGE(Comparativo!$O$6:$O$15,A16),Comparativo!$O$6:$O$15,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$B$6:$B$14,MATCH(LARGE(Comparativo!$O$6:$O$14,A16),Comparativo!$O$6:$O$14,0)),"")</f>
         <v/>
       </c>
       <c r="D16" s="18">
-        <f>IFERROR(INDEX(Comparativo!$I$6:$I$15,MATCH(LARGE(Comparativo!$O$6:$O$15,A16),Comparativo!$O$6:$O$15,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$I$6:$I$14,MATCH(LARGE(Comparativo!$O$6:$O$14,A16),Comparativo!$O$6:$O$14,0)),"")</f>
         <v/>
       </c>
       <c r="E16" s="18">
-        <f>IFERROR(INDEX(Comparativo!$J$6:$J$15,MATCH(LARGE(Comparativo!$O$6:$O$15,A16),Comparativo!$O$6:$O$15,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$J$6:$J$14,MATCH(LARGE(Comparativo!$O$6:$O$14,A16),Comparativo!$O$6:$O$14,0)),"")</f>
         <v/>
       </c>
       <c r="F16" s="18">
-        <f>IFERROR(INDEX(Comparativo!$K$6:$K$15,MATCH(LARGE(Comparativo!$O$6:$O$15,A16),Comparativo!$O$6:$O$15,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$K$6:$K$14,MATCH(LARGE(Comparativo!$O$6:$O$14,A16),Comparativo!$O$6:$O$14,0)),"")</f>
         <v/>
       </c>
       <c r="G16" s="19">
@@ -1389,23 +1389,23 @@
         <v>5</v>
       </c>
       <c r="B17" s="17">
-        <f>IFERROR(INDEX(Comparativo!$D$6:$D$15,MATCH(LARGE(Comparativo!$O$6:$O$15,A17),Comparativo!$O$6:$O$15,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$D$6:$D$14,MATCH(LARGE(Comparativo!$O$6:$O$14,A17),Comparativo!$O$6:$O$14,0)),"")</f>
         <v/>
       </c>
       <c r="C17" s="17">
-        <f>IFERROR(INDEX(Comparativo!$B$6:$B$15,MATCH(LARGE(Comparativo!$O$6:$O$15,A17),Comparativo!$O$6:$O$15,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$B$6:$B$14,MATCH(LARGE(Comparativo!$O$6:$O$14,A17),Comparativo!$O$6:$O$14,0)),"")</f>
         <v/>
       </c>
       <c r="D17" s="18">
-        <f>IFERROR(INDEX(Comparativo!$I$6:$I$15,MATCH(LARGE(Comparativo!$O$6:$O$15,A17),Comparativo!$O$6:$O$15,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$I$6:$I$14,MATCH(LARGE(Comparativo!$O$6:$O$14,A17),Comparativo!$O$6:$O$14,0)),"")</f>
         <v/>
       </c>
       <c r="E17" s="18">
-        <f>IFERROR(INDEX(Comparativo!$J$6:$J$15,MATCH(LARGE(Comparativo!$O$6:$O$15,A17),Comparativo!$O$6:$O$15,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$J$6:$J$14,MATCH(LARGE(Comparativo!$O$6:$O$14,A17),Comparativo!$O$6:$O$14,0)),"")</f>
         <v/>
       </c>
       <c r="F17" s="18">
-        <f>IFERROR(INDEX(Comparativo!$K$6:$K$15,MATCH(LARGE(Comparativo!$O$6:$O$15,A17),Comparativo!$O$6:$O$15,0)),"")</f>
+        <f>IFERROR(INDEX(Comparativo!$K$6:$K$14,MATCH(LARGE(Comparativo!$O$6:$O$14,A17),Comparativo!$O$6:$O$14,0)),"")</f>
         <v/>
       </c>
       <c r="G17" s="19">
@@ -1429,7 +1429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P29"/>
+  <dimension ref="A1:P27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2161,123 +2161,57 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="24">
-        <f>Planejado!A14</f>
-        <v/>
-      </c>
-      <c r="B15" s="24">
-        <f>Planejado!B14</f>
-        <v/>
-      </c>
-      <c r="C15" s="24">
-        <f>Planejado!C14</f>
-        <v/>
-      </c>
-      <c r="D15" s="25">
-        <f>Planejado!D14</f>
-        <v/>
-      </c>
-      <c r="E15" s="24">
-        <f>Planejado!G14</f>
-        <v/>
-      </c>
-      <c r="F15" s="26">
-        <f>INDEX(Planejado!$H14:$S14,$D$3)</f>
-        <v/>
-      </c>
-      <c r="G15" s="26">
-        <f>INDEX(Realizado!$H14:$S14,$D$3)</f>
-        <v/>
-      </c>
-      <c r="H15" s="26">
-        <f>G15-F15</f>
-        <v/>
-      </c>
-      <c r="I15" s="26">
-        <f>SUMPRODUCT((COLUMN(Planejado!$H$4:$S$4)-COLUMN(Planejado!$H$4)+1&lt;=$D$3)*Planejado!$H14:$S14)</f>
-        <v/>
-      </c>
-      <c r="J15" s="26">
-        <f>SUMPRODUCT((COLUMN(Realizado!$H$4:$S$4)-COLUMN(Realizado!$H$4)+1&lt;=$D$3)*Realizado!$H14:$S14)</f>
-        <v/>
-      </c>
-      <c r="K15" s="26">
-        <f>J15-I15</f>
-        <v/>
-      </c>
-      <c r="L15" s="27">
-        <f>IFERROR(K15/I15,"")</f>
-        <v/>
-      </c>
-      <c r="M15" s="27">
-        <f>IFERROR(J15/I15,"")</f>
-        <v/>
-      </c>
-      <c r="N15" s="28">
-        <f>IF(P15=0,"Sem lançamento",IF(AND(I15=0,J15=0),"—",IF(I15=0,"Não orçado",IF(K15&gt;0.05*I15,"Acima do orçado",IF(K15&lt;-0.05*I15,"Abaixo do orçado","Dentro do orçado")))))</f>
-        <v/>
-      </c>
-      <c r="O15" s="23">
-        <f>IF(K15&gt;1,K15+ROW()/1000000,"")</f>
-        <v/>
-      </c>
-      <c r="P15" s="29">
-        <f>SUMPRODUCT((COLUMN(Realizado!$H$4:$S$4)-COLUMN(Realizado!$H$4)+1&lt;=$D$3)*(Realizado!$H14:$S14&lt;&gt;""))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="30" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="30" t="inlineStr">
         <is>
           <t>TOTAL GERAL</t>
         </is>
       </c>
-      <c r="B29" s="30" t="n"/>
-      <c r="C29" s="30" t="n"/>
-      <c r="D29" s="30" t="n"/>
-      <c r="E29" s="30" t="n"/>
-      <c r="F29" s="31">
-        <f>SUM(F6:F15)</f>
-        <v/>
-      </c>
-      <c r="G29" s="31">
-        <f>SUM(G6:G15)</f>
-        <v/>
-      </c>
-      <c r="H29" s="31">
-        <f>SUM(H6:H15)</f>
-        <v/>
-      </c>
-      <c r="I29" s="31">
-        <f>SUM(I6:I15)</f>
-        <v/>
-      </c>
-      <c r="J29" s="31">
-        <f>SUM(J6:J15)</f>
-        <v/>
-      </c>
-      <c r="K29" s="31">
-        <f>SUM(K6:K15)</f>
-        <v/>
-      </c>
-      <c r="L29" s="32">
-        <f>IFERROR(K29/I29,"")</f>
-        <v/>
-      </c>
-      <c r="M29" s="32">
-        <f>IFERROR(J29/I29,"")</f>
-        <v/>
-      </c>
-      <c r="N29" s="30" t="n"/>
+      <c r="B27" s="30" t="n"/>
+      <c r="C27" s="30" t="n"/>
+      <c r="D27" s="30" t="n"/>
+      <c r="E27" s="30" t="n"/>
+      <c r="F27" s="31">
+        <f>SUM(F6:F14)</f>
+        <v/>
+      </c>
+      <c r="G27" s="31">
+        <f>SUM(G6:G14)</f>
+        <v/>
+      </c>
+      <c r="H27" s="31">
+        <f>SUM(H6:H14)</f>
+        <v/>
+      </c>
+      <c r="I27" s="31">
+        <f>SUM(I6:I14)</f>
+        <v/>
+      </c>
+      <c r="J27" s="31">
+        <f>SUM(J6:J14)</f>
+        <v/>
+      </c>
+      <c r="K27" s="31">
+        <f>SUM(K6:K14)</f>
+        <v/>
+      </c>
+      <c r="L27" s="32">
+        <f>IFERROR(K27/I27,"")</f>
+        <v/>
+      </c>
+      <c r="M27" s="32">
+        <f>IFERROR(J27/I27,"")</f>
+        <v/>
+      </c>
+      <c r="N27" s="30" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A5:N15"/>
+  <autoFilter ref="A5:N14"/>
   <mergeCells count="2">
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
-  <conditionalFormatting sqref="H6:H15">
+  <conditionalFormatting sqref="H6:H14">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -2285,7 +2219,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K6:K15">
+  <conditionalFormatting sqref="K6:K14">
     <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -2308,7 +2242,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T15"/>
+  <dimension ref="A1:T14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2544,12 +2478,12 @@
       </c>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>Geovanna — salário bruto</t>
+          <t>Geovanna</t>
         </is>
       </c>
       <c r="E6" s="25" t="inlineStr">
         <is>
-          <t>Analista Administrativo</t>
+          <t>Analista Administrativo — orçada pelo custo total (encargos de folha + benefícios). Salário bruto informado: R$ 2.886,91/mês</t>
         </is>
       </c>
       <c r="F6" s="24" t="inlineStr">
@@ -2563,40 +2497,40 @@
         </is>
       </c>
       <c r="H6" s="26" t="n">
-        <v>2886.91</v>
+        <v>4825.515</v>
       </c>
       <c r="I6" s="26" t="n">
-        <v>2886.91</v>
+        <v>4825.515</v>
       </c>
       <c r="J6" s="26" t="n">
-        <v>2886.91</v>
+        <v>4825.515</v>
       </c>
       <c r="K6" s="26" t="n">
-        <v>2886.91</v>
+        <v>4825.515</v>
       </c>
       <c r="L6" s="26" t="n">
-        <v>2886.91</v>
+        <v>4825.515</v>
       </c>
       <c r="M6" s="26" t="n">
-        <v>2886.91</v>
+        <v>4825.515</v>
       </c>
       <c r="N6" s="26" t="n">
-        <v>2886.91</v>
+        <v>4825.515</v>
       </c>
       <c r="O6" s="26" t="n">
-        <v>2886.91</v>
+        <v>4825.515</v>
       </c>
       <c r="P6" s="26" t="n">
-        <v>2886.91</v>
+        <v>4825.515</v>
       </c>
       <c r="Q6" s="26" t="n">
-        <v>2886.91</v>
+        <v>4825.515</v>
       </c>
       <c r="R6" s="26" t="n">
-        <v>2886.91</v>
+        <v>4825.515</v>
       </c>
       <c r="S6" s="26" t="n">
-        <v>2886.91</v>
+        <v>4825.515</v>
       </c>
       <c r="T6" s="33">
         <f>SUM(H6:S6)</f>
@@ -2606,7 +2540,7 @@
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="24" t="inlineStr">
         <is>
-          <t>JUR-E02B</t>
+          <t>JUR-E03</t>
         </is>
       </c>
       <c r="B7" s="24" t="inlineStr">
@@ -2621,59 +2555,59 @@
       </c>
       <c r="D7" s="25" t="inlineStr">
         <is>
-          <t>Geovanna — encargos e benefícios</t>
+          <t>Thamar Victória</t>
         </is>
       </c>
       <c r="E7" s="25" t="inlineStr">
         <is>
-          <t>INSS patronal, FGTS, provisões de 13º e férias, benefícios — PREENCHER</t>
+          <t>Advogada — reajuste permanente de R$ 5.000 para R$ 5.500 (revisado a partir de out/26)</t>
         </is>
       </c>
       <c r="F7" s="24" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>PJ</t>
         </is>
       </c>
       <c r="G7" s="24" t="inlineStr">
         <is>
-          <t>Encargos e Benefícios - CLT</t>
+          <t>Pessoal - PJ</t>
         </is>
       </c>
       <c r="H7" s="26" t="n">
-        <v>1938.605</v>
+        <v>5000</v>
       </c>
       <c r="I7" s="26" t="n">
-        <v>1938.605</v>
+        <v>5000</v>
       </c>
       <c r="J7" s="26" t="n">
-        <v>1938.605</v>
+        <v>5000</v>
       </c>
       <c r="K7" s="26" t="n">
-        <v>1938.605</v>
+        <v>5000</v>
       </c>
       <c r="L7" s="26" t="n">
-        <v>1938.605</v>
+        <v>5000</v>
       </c>
       <c r="M7" s="26" t="n">
-        <v>1938.605</v>
+        <v>5000</v>
       </c>
       <c r="N7" s="26" t="n">
-        <v>1938.605</v>
+        <v>5000</v>
       </c>
       <c r="O7" s="26" t="n">
-        <v>1938.605</v>
+        <v>5000</v>
       </c>
       <c r="P7" s="26" t="n">
-        <v>1938.605</v>
+        <v>5000</v>
       </c>
       <c r="Q7" s="26" t="n">
-        <v>1938.605</v>
+        <v>5500</v>
       </c>
       <c r="R7" s="26" t="n">
-        <v>1938.605</v>
+        <v>5500</v>
       </c>
       <c r="S7" s="26" t="n">
-        <v>1938.605</v>
+        <v>5500</v>
       </c>
       <c r="T7" s="33">
         <f>SUM(H7:S7)</f>
@@ -2683,7 +2617,7 @@
     <row r="8" ht="26" customHeight="1">
       <c r="A8" s="24" t="inlineStr">
         <is>
-          <t>JUR-E03</t>
+          <t>JUR-D01</t>
         </is>
       </c>
       <c r="B8" s="24" t="inlineStr">
@@ -2693,64 +2627,60 @@
       </c>
       <c r="C8" s="24" t="inlineStr">
         <is>
-          <t>Equipe</t>
+          <t>Despesas</t>
         </is>
       </c>
       <c r="D8" s="25" t="inlineStr">
         <is>
-          <t>Thamar Victória</t>
+          <t>JUSFY</t>
         </is>
       </c>
       <c r="E8" s="25" t="inlineStr">
         <is>
-          <t>Advogada — reajuste permanente de R$ 5.000 para R$ 5.500 (revisado a partir de out/26)</t>
-        </is>
-      </c>
-      <c r="F8" s="24" t="inlineStr">
-        <is>
-          <t>PJ</t>
-        </is>
-      </c>
+          <t>Fase de teste com objetivo de eliminar o Astrea</t>
+        </is>
+      </c>
+      <c r="F8" s="24" t="inlineStr"/>
       <c r="G8" s="24" t="inlineStr">
         <is>
-          <t>Pessoal - PJ</t>
+          <t>Licenças de Softwares</t>
         </is>
       </c>
       <c r="H8" s="26" t="n">
-        <v>5000</v>
+        <v>100</v>
       </c>
       <c r="I8" s="26" t="n">
-        <v>5000</v>
+        <v>100</v>
       </c>
       <c r="J8" s="26" t="n">
-        <v>5000</v>
+        <v>100</v>
       </c>
       <c r="K8" s="26" t="n">
-        <v>5000</v>
+        <v>100</v>
       </c>
       <c r="L8" s="26" t="n">
-        <v>5000</v>
+        <v>100</v>
       </c>
       <c r="M8" s="26" t="n">
-        <v>5000</v>
+        <v>100</v>
       </c>
       <c r="N8" s="26" t="n">
-        <v>5000</v>
+        <v>100</v>
       </c>
       <c r="O8" s="26" t="n">
-        <v>5000</v>
+        <v>100</v>
       </c>
       <c r="P8" s="26" t="n">
-        <v>5000</v>
+        <v>100</v>
       </c>
       <c r="Q8" s="26" t="n">
-        <v>5500</v>
+        <v>100</v>
       </c>
       <c r="R8" s="26" t="n">
-        <v>5500</v>
+        <v>100</v>
       </c>
       <c r="S8" s="26" t="n">
-        <v>5500</v>
+        <v>100</v>
       </c>
       <c r="T8" s="33">
         <f>SUM(H8:S8)</f>
@@ -2760,7 +2690,7 @@
     <row r="9" ht="26" customHeight="1">
       <c r="A9" s="24" t="inlineStr">
         <is>
-          <t>JUR-D01</t>
+          <t>JUR-D02</t>
         </is>
       </c>
       <c r="B9" s="24" t="inlineStr">
@@ -2775,14 +2705,10 @@
       </c>
       <c r="D9" s="25" t="inlineStr">
         <is>
-          <t>JUSFY</t>
-        </is>
-      </c>
-      <c r="E9" s="25" t="inlineStr">
-        <is>
-          <t>Fase de teste com objetivo de eliminar o Astrea</t>
-        </is>
-      </c>
+          <t>JUSBRASIL</t>
+        </is>
+      </c>
+      <c r="E9" s="25" t="inlineStr"/>
       <c r="F9" s="24" t="inlineStr"/>
       <c r="G9" s="24" t="inlineStr">
         <is>
@@ -2790,40 +2716,40 @@
         </is>
       </c>
       <c r="H9" s="26" t="n">
-        <v>100</v>
+        <v>104.9</v>
       </c>
       <c r="I9" s="26" t="n">
-        <v>100</v>
+        <v>104.9</v>
       </c>
       <c r="J9" s="26" t="n">
-        <v>100</v>
+        <v>104.9</v>
       </c>
       <c r="K9" s="26" t="n">
-        <v>100</v>
+        <v>104.9</v>
       </c>
       <c r="L9" s="26" t="n">
-        <v>100</v>
+        <v>104.9</v>
       </c>
       <c r="M9" s="26" t="n">
-        <v>100</v>
+        <v>104.9</v>
       </c>
       <c r="N9" s="26" t="n">
-        <v>100</v>
+        <v>104.9</v>
       </c>
       <c r="O9" s="26" t="n">
-        <v>100</v>
+        <v>104.9</v>
       </c>
       <c r="P9" s="26" t="n">
-        <v>100</v>
+        <v>104.9</v>
       </c>
       <c r="Q9" s="26" t="n">
-        <v>100</v>
+        <v>104.9</v>
       </c>
       <c r="R9" s="26" t="n">
-        <v>100</v>
+        <v>104.9</v>
       </c>
       <c r="S9" s="26" t="n">
-        <v>100</v>
+        <v>104.9</v>
       </c>
       <c r="T9" s="33">
         <f>SUM(H9:S9)</f>
@@ -2833,7 +2759,7 @@
     <row r="10" ht="26" customHeight="1">
       <c r="A10" s="24" t="inlineStr">
         <is>
-          <t>JUR-D02</t>
+          <t>JUR-D03</t>
         </is>
       </c>
       <c r="B10" s="24" t="inlineStr">
@@ -2848,10 +2774,14 @@
       </c>
       <c r="D10" s="25" t="inlineStr">
         <is>
-          <t>JUSBRASIL</t>
-        </is>
-      </c>
-      <c r="E10" s="25" t="inlineStr"/>
+          <t>ASTREA</t>
+        </is>
+      </c>
+      <c r="E10" s="25" t="inlineStr">
+        <is>
+          <t>Cancelado — realizado zerado desde mai/26</t>
+        </is>
+      </c>
       <c r="F10" s="24" t="inlineStr"/>
       <c r="G10" s="24" t="inlineStr">
         <is>
@@ -2859,40 +2789,40 @@
         </is>
       </c>
       <c r="H10" s="26" t="n">
-        <v>104.9</v>
+        <v>112.07</v>
       </c>
       <c r="I10" s="26" t="n">
-        <v>104.9</v>
+        <v>112.07</v>
       </c>
       <c r="J10" s="26" t="n">
-        <v>104.9</v>
+        <v>112.07</v>
       </c>
       <c r="K10" s="26" t="n">
-        <v>104.9</v>
+        <v>112.07</v>
       </c>
       <c r="L10" s="26" t="n">
-        <v>104.9</v>
+        <v>112.07</v>
       </c>
       <c r="M10" s="26" t="n">
-        <v>104.9</v>
+        <v>112.07</v>
       </c>
       <c r="N10" s="26" t="n">
-        <v>104.9</v>
+        <v>112.07</v>
       </c>
       <c r="O10" s="26" t="n">
-        <v>104.9</v>
+        <v>112.07</v>
       </c>
       <c r="P10" s="26" t="n">
-        <v>104.9</v>
+        <v>112.07</v>
       </c>
       <c r="Q10" s="26" t="n">
-        <v>104.9</v>
+        <v>112.07</v>
       </c>
       <c r="R10" s="26" t="n">
-        <v>104.9</v>
+        <v>112.07</v>
       </c>
       <c r="S10" s="26" t="n">
-        <v>104.9</v>
+        <v>112.07</v>
       </c>
       <c r="T10" s="33">
         <f>SUM(H10:S10)</f>
@@ -2902,7 +2832,7 @@
     <row r="11" ht="26" customHeight="1">
       <c r="A11" s="24" t="inlineStr">
         <is>
-          <t>JUR-D03</t>
+          <t>JUR-D04</t>
         </is>
       </c>
       <c r="B11" s="24" t="inlineStr">
@@ -2917,14 +2847,10 @@
       </c>
       <c r="D11" s="25" t="inlineStr">
         <is>
-          <t>ASTREA</t>
-        </is>
-      </c>
-      <c r="E11" s="25" t="inlineStr">
-        <is>
-          <t>Cancelado — realizado zerado desde mai/26</t>
-        </is>
-      </c>
+          <t>LEME</t>
+        </is>
+      </c>
+      <c r="E11" s="25" t="inlineStr"/>
       <c r="F11" s="24" t="inlineStr"/>
       <c r="G11" s="24" t="inlineStr">
         <is>
@@ -2932,40 +2858,40 @@
         </is>
       </c>
       <c r="H11" s="26" t="n">
-        <v>112.07</v>
+        <v>1030</v>
       </c>
       <c r="I11" s="26" t="n">
-        <v>112.07</v>
+        <v>1030</v>
       </c>
       <c r="J11" s="26" t="n">
-        <v>112.07</v>
+        <v>1030</v>
       </c>
       <c r="K11" s="26" t="n">
-        <v>112.07</v>
+        <v>1030</v>
       </c>
       <c r="L11" s="26" t="n">
-        <v>112.07</v>
+        <v>1030</v>
       </c>
       <c r="M11" s="26" t="n">
-        <v>112.07</v>
+        <v>1030</v>
       </c>
       <c r="N11" s="26" t="n">
-        <v>112.07</v>
+        <v>1030</v>
       </c>
       <c r="O11" s="26" t="n">
-        <v>112.07</v>
+        <v>1030</v>
       </c>
       <c r="P11" s="26" t="n">
-        <v>112.07</v>
+        <v>1030</v>
       </c>
       <c r="Q11" s="26" t="n">
-        <v>112.07</v>
+        <v>1030</v>
       </c>
       <c r="R11" s="26" t="n">
-        <v>112.07</v>
+        <v>1030</v>
       </c>
       <c r="S11" s="26" t="n">
-        <v>112.07</v>
+        <v>1030</v>
       </c>
       <c r="T11" s="33">
         <f>SUM(H11:S11)</f>
@@ -2975,7 +2901,7 @@
     <row r="12" ht="26" customHeight="1">
       <c r="A12" s="24" t="inlineStr">
         <is>
-          <t>JUR-D04</t>
+          <t>JUR-D05</t>
         </is>
       </c>
       <c r="B12" s="24" t="inlineStr">
@@ -2990,51 +2916,51 @@
       </c>
       <c r="D12" s="25" t="inlineStr">
         <is>
-          <t>LEME</t>
+          <t>Cursos / Eventos / Network</t>
         </is>
       </c>
       <c r="E12" s="25" t="inlineStr"/>
       <c r="F12" s="24" t="inlineStr"/>
       <c r="G12" s="24" t="inlineStr">
         <is>
-          <t>Licenças de Softwares</t>
+          <t>Custeio de Treinamento</t>
         </is>
       </c>
       <c r="H12" s="26" t="n">
-        <v>1030</v>
+        <v>1000</v>
       </c>
       <c r="I12" s="26" t="n">
-        <v>1030</v>
+        <v>1000</v>
       </c>
       <c r="J12" s="26" t="n">
-        <v>1030</v>
+        <v>1000</v>
       </c>
       <c r="K12" s="26" t="n">
-        <v>1030</v>
+        <v>1000</v>
       </c>
       <c r="L12" s="26" t="n">
-        <v>1030</v>
+        <v>1000</v>
       </c>
       <c r="M12" s="26" t="n">
-        <v>1030</v>
+        <v>1000</v>
       </c>
       <c r="N12" s="26" t="n">
-        <v>1030</v>
+        <v>1000</v>
       </c>
       <c r="O12" s="26" t="n">
-        <v>1030</v>
+        <v>1000</v>
       </c>
       <c r="P12" s="26" t="n">
-        <v>1030</v>
+        <v>1000</v>
       </c>
       <c r="Q12" s="26" t="n">
-        <v>1030</v>
+        <v>1000</v>
       </c>
       <c r="R12" s="26" t="n">
-        <v>1030</v>
+        <v>1000</v>
       </c>
       <c r="S12" s="26" t="n">
-        <v>1030</v>
+        <v>1000</v>
       </c>
       <c r="T12" s="33">
         <f>SUM(H12:S12)</f>
@@ -3044,7 +2970,7 @@
     <row r="13" ht="26" customHeight="1">
       <c r="A13" s="24" t="inlineStr">
         <is>
-          <t>JUR-D05</t>
+          <t>JUR-D06</t>
         </is>
       </c>
       <c r="B13" s="24" t="inlineStr">
@@ -3059,197 +2985,128 @@
       </c>
       <c r="D13" s="25" t="inlineStr">
         <is>
-          <t>Cursos / Eventos / Network</t>
-        </is>
-      </c>
-      <c r="E13" s="25" t="inlineStr"/>
+          <t>Bonificações trimestrais/semestrais do time</t>
+        </is>
+      </c>
+      <c r="E13" s="25" t="inlineStr">
+        <is>
+          <t>Participação em projetos e atingimento de resultados — CONFIRMAR se houve parcela no 1º quadrimestre</t>
+        </is>
+      </c>
       <c r="F13" s="24" t="inlineStr"/>
       <c r="G13" s="24" t="inlineStr">
         <is>
-          <t>Custeio de Treinamento</t>
+          <t>Prêmios</t>
         </is>
       </c>
       <c r="H13" s="26" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="I13" s="26" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="J13" s="26" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="K13" s="26" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="L13" s="26" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="M13" s="26" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="N13" s="26" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="O13" s="26" t="n">
-        <v>1000</v>
+        <v>10293.6</v>
       </c>
       <c r="P13" s="26" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="Q13" s="26" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="R13" s="26" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="S13" s="26" t="n">
-        <v>1000</v>
+        <v>12867</v>
       </c>
       <c r="T13" s="33">
         <f>SUM(H13:S13)</f>
         <v/>
       </c>
     </row>
-    <row r="14" ht="26" customHeight="1">
-      <c r="A14" s="24" t="inlineStr">
-        <is>
-          <t>JUR-D06</t>
-        </is>
-      </c>
-      <c r="B14" s="24" t="inlineStr">
-        <is>
-          <t>Jurídico</t>
-        </is>
-      </c>
-      <c r="C14" s="24" t="inlineStr">
-        <is>
-          <t>Despesas</t>
-        </is>
-      </c>
-      <c r="D14" s="25" t="inlineStr">
-        <is>
-          <t>Bonificações trimestrais/semestrais do time</t>
-        </is>
-      </c>
-      <c r="E14" s="25" t="inlineStr">
-        <is>
-          <t>Participação em projetos e atingimento de resultados — CONFIRMAR se houve parcela no 1º quadrimestre</t>
-        </is>
-      </c>
-      <c r="F14" s="24" t="inlineStr"/>
-      <c r="G14" s="24" t="inlineStr">
-        <is>
-          <t>Prêmios</t>
-        </is>
-      </c>
-      <c r="H14" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" s="26" t="n">
-        <v>10293.6</v>
-      </c>
-      <c r="P14" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q14" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="R14" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="S14" s="26" t="n">
-        <v>12867</v>
-      </c>
-      <c r="T14" s="33">
-        <f>SUM(H14:S14)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="30" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="30" t="inlineStr">
         <is>
           <t>TOTAL GERAL</t>
         </is>
       </c>
-      <c r="B15" s="30" t="n"/>
-      <c r="C15" s="30" t="n"/>
-      <c r="D15" s="30" t="n"/>
-      <c r="E15" s="30" t="n"/>
-      <c r="F15" s="30" t="n"/>
-      <c r="G15" s="30" t="n"/>
-      <c r="H15" s="31">
-        <f>SUM(H5:H14)</f>
-        <v/>
-      </c>
-      <c r="I15" s="31">
-        <f>SUM(I5:I14)</f>
-        <v/>
-      </c>
-      <c r="J15" s="31">
-        <f>SUM(J5:J14)</f>
-        <v/>
-      </c>
-      <c r="K15" s="31">
-        <f>SUM(K5:K14)</f>
-        <v/>
-      </c>
-      <c r="L15" s="31">
-        <f>SUM(L5:L14)</f>
-        <v/>
-      </c>
-      <c r="M15" s="31">
-        <f>SUM(M5:M14)</f>
-        <v/>
-      </c>
-      <c r="N15" s="31">
-        <f>SUM(N5:N14)</f>
-        <v/>
-      </c>
-      <c r="O15" s="31">
-        <f>SUM(O5:O14)</f>
-        <v/>
-      </c>
-      <c r="P15" s="31">
-        <f>SUM(P5:P14)</f>
-        <v/>
-      </c>
-      <c r="Q15" s="31">
-        <f>SUM(Q5:Q14)</f>
-        <v/>
-      </c>
-      <c r="R15" s="31">
-        <f>SUM(R5:R14)</f>
-        <v/>
-      </c>
-      <c r="S15" s="31">
-        <f>SUM(S5:S14)</f>
-        <v/>
-      </c>
-      <c r="T15" s="31">
-        <f>SUM(T5:T14)</f>
+      <c r="B14" s="30" t="n"/>
+      <c r="C14" s="30" t="n"/>
+      <c r="D14" s="30" t="n"/>
+      <c r="E14" s="30" t="n"/>
+      <c r="F14" s="30" t="n"/>
+      <c r="G14" s="30" t="n"/>
+      <c r="H14" s="31">
+        <f>SUM(H5:H13)</f>
+        <v/>
+      </c>
+      <c r="I14" s="31">
+        <f>SUM(I5:I13)</f>
+        <v/>
+      </c>
+      <c r="J14" s="31">
+        <f>SUM(J5:J13)</f>
+        <v/>
+      </c>
+      <c r="K14" s="31">
+        <f>SUM(K5:K13)</f>
+        <v/>
+      </c>
+      <c r="L14" s="31">
+        <f>SUM(L5:L13)</f>
+        <v/>
+      </c>
+      <c r="M14" s="31">
+        <f>SUM(M5:M13)</f>
+        <v/>
+      </c>
+      <c r="N14" s="31">
+        <f>SUM(N5:N13)</f>
+        <v/>
+      </c>
+      <c r="O14" s="31">
+        <f>SUM(O5:O13)</f>
+        <v/>
+      </c>
+      <c r="P14" s="31">
+        <f>SUM(P5:P13)</f>
+        <v/>
+      </c>
+      <c r="Q14" s="31">
+        <f>SUM(Q5:Q13)</f>
+        <v/>
+      </c>
+      <c r="R14" s="31">
+        <f>SUM(R5:R13)</f>
+        <v/>
+      </c>
+      <c r="S14" s="31">
+        <f>SUM(S5:S13)</f>
+        <v/>
+      </c>
+      <c r="T14" s="31">
+        <f>SUM(T5:T13)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:T14"/>
+  <autoFilter ref="A4:T13"/>
   <mergeCells count="2">
     <mergeCell ref="A1:T1"/>
     <mergeCell ref="A2:T2"/>
@@ -3264,7 +3121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V15"/>
+  <dimension ref="A1:V14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3508,28 +3365,18 @@
       <c r="I6" s="37" t="n"/>
       <c r="J6" s="37" t="n"/>
       <c r="K6" s="37" t="n"/>
-      <c r="L6" s="37" t="n">
-        <v>2886.91</v>
-      </c>
-      <c r="M6" s="37" t="n">
-        <v>2886.91</v>
-      </c>
-      <c r="N6" s="37" t="n">
-        <v>2886.91</v>
-      </c>
+      <c r="L6" s="37" t="n"/>
+      <c r="M6" s="37" t="n"/>
+      <c r="N6" s="37" t="n"/>
       <c r="O6" s="37" t="n"/>
       <c r="T6" s="33">
         <f>SUM(H6:S6)</f>
         <v/>
       </c>
-      <c r="U6" s="38" t="inlineStr">
-        <is>
-          <t>Gestora, 05/08/26</t>
-        </is>
-      </c>
+      <c r="U6" s="38" t="n"/>
       <c r="V6" s="38" t="inlineStr">
         <is>
-          <t>Salário bruto</t>
+          <t>PREENCHER com o CUSTO TOTAL. Bruto informado: R$ 2.886,91/mês — faltam encargos e benefícios</t>
         </is>
       </c>
     </row>
@@ -3566,18 +3413,28 @@
       <c r="I7" s="37" t="n"/>
       <c r="J7" s="37" t="n"/>
       <c r="K7" s="37" t="n"/>
-      <c r="L7" s="37" t="n"/>
-      <c r="M7" s="37" t="n"/>
-      <c r="N7" s="37" t="n"/>
+      <c r="L7" s="37" t="n">
+        <v>5500</v>
+      </c>
+      <c r="M7" s="37" t="n">
+        <v>5500</v>
+      </c>
+      <c r="N7" s="37" t="n">
+        <v>5500</v>
+      </c>
       <c r="O7" s="37" t="n"/>
       <c r="T7" s="33">
         <f>SUM(H7:S7)</f>
         <v/>
       </c>
-      <c r="U7" s="38" t="n"/>
+      <c r="U7" s="38" t="inlineStr">
+        <is>
+          <t>Gestora, 05/08/26</t>
+        </is>
+      </c>
       <c r="V7" s="38" t="inlineStr">
         <is>
-          <t>PREENCHER — encargos e benefícios sobre o bruto</t>
+          <t>Reajuste permanente aplicado desde mai/26</t>
         </is>
       </c>
     </row>
@@ -3615,13 +3472,13 @@
       <c r="J8" s="37" t="n"/>
       <c r="K8" s="37" t="n"/>
       <c r="L8" s="37" t="n">
-        <v>5500</v>
+        <v>0</v>
       </c>
       <c r="M8" s="37" t="n">
-        <v>5500</v>
+        <v>0</v>
       </c>
       <c r="N8" s="37" t="n">
-        <v>5500</v>
+        <v>0</v>
       </c>
       <c r="O8" s="37" t="n"/>
       <c r="T8" s="33">
@@ -3635,7 +3492,7 @@
       </c>
       <c r="V8" s="38" t="inlineStr">
         <is>
-          <t>Reajuste permanente aplicado desde mai/26</t>
+          <t>Ainda não iniciado — sem cobrança</t>
         </is>
       </c>
     </row>
@@ -3673,13 +3530,13 @@
       <c r="J9" s="37" t="n"/>
       <c r="K9" s="37" t="n"/>
       <c r="L9" s="37" t="n">
-        <v>0</v>
+        <v>136</v>
       </c>
       <c r="M9" s="37" t="n">
-        <v>0</v>
+        <v>136</v>
       </c>
       <c r="N9" s="37" t="n">
-        <v>0</v>
+        <v>136</v>
       </c>
       <c r="O9" s="37" t="n"/>
       <c r="T9" s="33">
@@ -3693,7 +3550,7 @@
       </c>
       <c r="V9" s="38" t="inlineStr">
         <is>
-          <t>Ainda não iniciado — sem cobrança</t>
+          <t>Acima do orçado (R$ 104,90) — conferir contrato</t>
         </is>
       </c>
     </row>
@@ -3731,13 +3588,13 @@
       <c r="J10" s="37" t="n"/>
       <c r="K10" s="37" t="n"/>
       <c r="L10" s="37" t="n">
-        <v>136</v>
+        <v>0</v>
       </c>
       <c r="M10" s="37" t="n">
-        <v>136</v>
+        <v>0</v>
       </c>
       <c r="N10" s="37" t="n">
-        <v>136</v>
+        <v>0</v>
       </c>
       <c r="O10" s="37" t="n"/>
       <c r="T10" s="33">
@@ -3751,7 +3608,7 @@
       </c>
       <c r="V10" s="38" t="inlineStr">
         <is>
-          <t>Acima do orçado (R$ 104,90) — conferir contrato</t>
+          <t>Cancelado — sem cobrança</t>
         </is>
       </c>
     </row>
@@ -3789,13 +3646,13 @@
       <c r="J11" s="37" t="n"/>
       <c r="K11" s="37" t="n"/>
       <c r="L11" s="37" t="n">
-        <v>0</v>
+        <v>970</v>
       </c>
       <c r="M11" s="37" t="n">
-        <v>0</v>
+        <v>970</v>
       </c>
       <c r="N11" s="37" t="n">
-        <v>0</v>
+        <v>970</v>
       </c>
       <c r="O11" s="37" t="n"/>
       <c r="T11" s="33">
@@ -3807,11 +3664,7 @@
           <t>Gestora, 05/08/26</t>
         </is>
       </c>
-      <c r="V11" s="38" t="inlineStr">
-        <is>
-          <t>Cancelado — sem cobrança</t>
-        </is>
-      </c>
+      <c r="V11" s="38" t="n"/>
     </row>
     <row r="12" ht="26" customHeight="1">
       <c r="A12" s="35">
@@ -3847,13 +3700,13 @@
       <c r="J12" s="37" t="n"/>
       <c r="K12" s="37" t="n"/>
       <c r="L12" s="37" t="n">
-        <v>970</v>
+        <v>0</v>
       </c>
       <c r="M12" s="37" t="n">
-        <v>970</v>
+        <v>0</v>
       </c>
       <c r="N12" s="37" t="n">
-        <v>970</v>
+        <v>0</v>
       </c>
       <c r="O12" s="37" t="n"/>
       <c r="T12" s="33">
@@ -3865,7 +3718,11 @@
           <t>Gestora, 05/08/26</t>
         </is>
       </c>
-      <c r="V12" s="38" t="n"/>
+      <c r="V12" s="38" t="inlineStr">
+        <is>
+          <t>Sem gasto no período</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="26" customHeight="1">
       <c r="A13" s="35">
@@ -3900,145 +3757,87 @@
       <c r="I13" s="37" t="n"/>
       <c r="J13" s="37" t="n"/>
       <c r="K13" s="37" t="n"/>
-      <c r="L13" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" s="37" t="n">
-        <v>0</v>
-      </c>
+      <c r="L13" s="37" t="n"/>
+      <c r="M13" s="37" t="n"/>
+      <c r="N13" s="37" t="n"/>
       <c r="O13" s="37" t="n"/>
       <c r="T13" s="33">
         <f>SUM(H13:S13)</f>
         <v/>
       </c>
-      <c r="U13" s="38" t="inlineStr">
-        <is>
-          <t>Gestora, 05/08/26</t>
-        </is>
-      </c>
+      <c r="U13" s="38" t="n"/>
       <c r="V13" s="38" t="inlineStr">
         <is>
-          <t>Sem gasto no período</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="26" customHeight="1">
-      <c r="A14" s="35">
-        <f>Planejado!A14</f>
-        <v/>
-      </c>
-      <c r="B14" s="35">
-        <f>Planejado!B14</f>
-        <v/>
-      </c>
-      <c r="C14" s="35">
-        <f>Planejado!C14</f>
-        <v/>
-      </c>
-      <c r="D14" s="36">
-        <f>Planejado!D14</f>
-        <v/>
-      </c>
-      <c r="E14" s="36">
-        <f>Planejado!E14</f>
-        <v/>
-      </c>
-      <c r="F14" s="35">
-        <f>Planejado!F14</f>
-        <v/>
-      </c>
-      <c r="G14" s="35">
-        <f>Planejado!G14</f>
-        <v/>
-      </c>
-      <c r="H14" s="37" t="n"/>
-      <c r="I14" s="37" t="n"/>
-      <c r="J14" s="37" t="n"/>
-      <c r="K14" s="37" t="n"/>
-      <c r="L14" s="37" t="n"/>
-      <c r="M14" s="37" t="n"/>
-      <c r="N14" s="37" t="n"/>
-      <c r="O14" s="37" t="n"/>
-      <c r="T14" s="33">
-        <f>SUM(H14:S14)</f>
-        <v/>
-      </c>
-      <c r="U14" s="38" t="n"/>
-      <c r="V14" s="38" t="inlineStr">
-        <is>
           <t>Bonificação de ago/26 a confirmar</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="39" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="39" t="inlineStr">
         <is>
           <t>TOTAL GERAL</t>
         </is>
       </c>
-      <c r="B15" s="39" t="n"/>
-      <c r="C15" s="39" t="n"/>
-      <c r="D15" s="39" t="n"/>
-      <c r="E15" s="39" t="n"/>
-      <c r="F15" s="39" t="n"/>
-      <c r="G15" s="39" t="n"/>
-      <c r="H15" s="40">
-        <f>SUM(H5:H14)</f>
-        <v/>
-      </c>
-      <c r="I15" s="40">
-        <f>SUM(I5:I14)</f>
-        <v/>
-      </c>
-      <c r="J15" s="40">
-        <f>SUM(J5:J14)</f>
-        <v/>
-      </c>
-      <c r="K15" s="40">
-        <f>SUM(K5:K14)</f>
-        <v/>
-      </c>
-      <c r="L15" s="40">
-        <f>SUM(L5:L14)</f>
-        <v/>
-      </c>
-      <c r="M15" s="40">
-        <f>SUM(M5:M14)</f>
-        <v/>
-      </c>
-      <c r="N15" s="40">
-        <f>SUM(N5:N14)</f>
-        <v/>
-      </c>
-      <c r="O15" s="40">
-        <f>SUM(O5:O14)</f>
-        <v/>
-      </c>
-      <c r="P15" s="40">
-        <f>SUM(P5:P14)</f>
-        <v/>
-      </c>
-      <c r="Q15" s="40">
-        <f>SUM(Q5:Q14)</f>
-        <v/>
-      </c>
-      <c r="R15" s="40">
-        <f>SUM(R5:R14)</f>
-        <v/>
-      </c>
-      <c r="S15" s="40">
-        <f>SUM(S5:S14)</f>
-        <v/>
-      </c>
-      <c r="T15" s="40">
-        <f>SUM(T5:T14)</f>
-        <v/>
-      </c>
-      <c r="U15" s="39" t="n"/>
-      <c r="V15" s="39" t="n"/>
+      <c r="B14" s="39" t="n"/>
+      <c r="C14" s="39" t="n"/>
+      <c r="D14" s="39" t="n"/>
+      <c r="E14" s="39" t="n"/>
+      <c r="F14" s="39" t="n"/>
+      <c r="G14" s="39" t="n"/>
+      <c r="H14" s="40">
+        <f>SUM(H5:H13)</f>
+        <v/>
+      </c>
+      <c r="I14" s="40">
+        <f>SUM(I5:I13)</f>
+        <v/>
+      </c>
+      <c r="J14" s="40">
+        <f>SUM(J5:J13)</f>
+        <v/>
+      </c>
+      <c r="K14" s="40">
+        <f>SUM(K5:K13)</f>
+        <v/>
+      </c>
+      <c r="L14" s="40">
+        <f>SUM(L5:L13)</f>
+        <v/>
+      </c>
+      <c r="M14" s="40">
+        <f>SUM(M5:M13)</f>
+        <v/>
+      </c>
+      <c r="N14" s="40">
+        <f>SUM(N5:N13)</f>
+        <v/>
+      </c>
+      <c r="O14" s="40">
+        <f>SUM(O5:O13)</f>
+        <v/>
+      </c>
+      <c r="P14" s="40">
+        <f>SUM(P5:P13)</f>
+        <v/>
+      </c>
+      <c r="Q14" s="40">
+        <f>SUM(Q5:Q13)</f>
+        <v/>
+      </c>
+      <c r="R14" s="40">
+        <f>SUM(R5:R13)</f>
+        <v/>
+      </c>
+      <c r="S14" s="40">
+        <f>SUM(S5:S13)</f>
+        <v/>
+      </c>
+      <c r="T14" s="40">
+        <f>SUM(T5:T13)</f>
+        <v/>
+      </c>
+      <c r="U14" s="39" t="n"/>
+      <c r="V14" s="39" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4131,11 +3930,11 @@
         </is>
       </c>
       <c r="B5" s="26">
-        <f>SUMIFS(Planejado!$H$5:$H$14,Planejado!$B$5:$B$14,"Jurídico")</f>
+        <f>SUMIFS(Planejado!$H$5:$H$13,Planejado!$B$5:$B$13,"Jurídico")</f>
         <v/>
       </c>
       <c r="C5" s="26">
-        <f>SUMIFS(Realizado!$H$5:$H$14,Realizado!$B$5:$B$14,"Jurídico")</f>
+        <f>SUMIFS(Realizado!$H$5:$H$13,Realizado!$B$5:$B$13,"Jurídico")</f>
         <v/>
       </c>
       <c r="D5" s="26">
@@ -4166,11 +3965,11 @@
         </is>
       </c>
       <c r="B6" s="43">
-        <f>SUMIFS(Planejado!$I$5:$I$14,Planejado!$B$5:$B$14,"Jurídico")</f>
+        <f>SUMIFS(Planejado!$I$5:$I$13,Planejado!$B$5:$B$13,"Jurídico")</f>
         <v/>
       </c>
       <c r="C6" s="43">
-        <f>SUMIFS(Realizado!$I$5:$I$14,Realizado!$B$5:$B$14,"Jurídico")</f>
+        <f>SUMIFS(Realizado!$I$5:$I$13,Realizado!$B$5:$B$13,"Jurídico")</f>
         <v/>
       </c>
       <c r="D6" s="43">
@@ -4201,11 +4000,11 @@
         </is>
       </c>
       <c r="B7" s="26">
-        <f>SUMIFS(Planejado!$J$5:$J$14,Planejado!$B$5:$B$14,"Jurídico")</f>
+        <f>SUMIFS(Planejado!$J$5:$J$13,Planejado!$B$5:$B$13,"Jurídico")</f>
         <v/>
       </c>
       <c r="C7" s="26">
-        <f>SUMIFS(Realizado!$J$5:$J$14,Realizado!$B$5:$B$14,"Jurídico")</f>
+        <f>SUMIFS(Realizado!$J$5:$J$13,Realizado!$B$5:$B$13,"Jurídico")</f>
         <v/>
       </c>
       <c r="D7" s="26">
@@ -4236,11 +4035,11 @@
         </is>
       </c>
       <c r="B8" s="43">
-        <f>SUMIFS(Planejado!$K$5:$K$14,Planejado!$B$5:$B$14,"Jurídico")</f>
+        <f>SUMIFS(Planejado!$K$5:$K$13,Planejado!$B$5:$B$13,"Jurídico")</f>
         <v/>
       </c>
       <c r="C8" s="43">
-        <f>SUMIFS(Realizado!$K$5:$K$14,Realizado!$B$5:$B$14,"Jurídico")</f>
+        <f>SUMIFS(Realizado!$K$5:$K$13,Realizado!$B$5:$B$13,"Jurídico")</f>
         <v/>
       </c>
       <c r="D8" s="43">
@@ -4271,11 +4070,11 @@
         </is>
       </c>
       <c r="B9" s="26">
-        <f>SUMIFS(Planejado!$L$5:$L$14,Planejado!$B$5:$B$14,"Jurídico")</f>
+        <f>SUMIFS(Planejado!$L$5:$L$13,Planejado!$B$5:$B$13,"Jurídico")</f>
         <v/>
       </c>
       <c r="C9" s="26">
-        <f>SUMIFS(Realizado!$L$5:$L$14,Realizado!$B$5:$B$14,"Jurídico")</f>
+        <f>SUMIFS(Realizado!$L$5:$L$13,Realizado!$B$5:$B$13,"Jurídico")</f>
         <v/>
       </c>
       <c r="D9" s="26">
@@ -4306,11 +4105,11 @@
         </is>
       </c>
       <c r="B10" s="43">
-        <f>SUMIFS(Planejado!$M$5:$M$14,Planejado!$B$5:$B$14,"Jurídico")</f>
+        <f>SUMIFS(Planejado!$M$5:$M$13,Planejado!$B$5:$B$13,"Jurídico")</f>
         <v/>
       </c>
       <c r="C10" s="43">
-        <f>SUMIFS(Realizado!$M$5:$M$14,Realizado!$B$5:$B$14,"Jurídico")</f>
+        <f>SUMIFS(Realizado!$M$5:$M$13,Realizado!$B$5:$B$13,"Jurídico")</f>
         <v/>
       </c>
       <c r="D10" s="43">
@@ -4341,11 +4140,11 @@
         </is>
       </c>
       <c r="B11" s="26">
-        <f>SUMIFS(Planejado!$N$5:$N$14,Planejado!$B$5:$B$14,"Jurídico")</f>
+        <f>SUMIFS(Planejado!$N$5:$N$13,Planejado!$B$5:$B$13,"Jurídico")</f>
         <v/>
       </c>
       <c r="C11" s="26">
-        <f>SUMIFS(Realizado!$N$5:$N$14,Realizado!$B$5:$B$14,"Jurídico")</f>
+        <f>SUMIFS(Realizado!$N$5:$N$13,Realizado!$B$5:$B$13,"Jurídico")</f>
         <v/>
       </c>
       <c r="D11" s="26">
@@ -4376,11 +4175,11 @@
         </is>
       </c>
       <c r="B12" s="43">
-        <f>SUMIFS(Planejado!$O$5:$O$14,Planejado!$B$5:$B$14,"Jurídico")</f>
+        <f>SUMIFS(Planejado!$O$5:$O$13,Planejado!$B$5:$B$13,"Jurídico")</f>
         <v/>
       </c>
       <c r="C12" s="43">
-        <f>SUMIFS(Realizado!$O$5:$O$14,Realizado!$B$5:$B$14,"Jurídico")</f>
+        <f>SUMIFS(Realizado!$O$5:$O$13,Realizado!$B$5:$B$13,"Jurídico")</f>
         <v/>
       </c>
       <c r="D12" s="43">
@@ -4411,11 +4210,11 @@
         </is>
       </c>
       <c r="B13" s="26">
-        <f>SUMIFS(Planejado!$P$5:$P$14,Planejado!$B$5:$B$14,"Jurídico")</f>
+        <f>SUMIFS(Planejado!$P$5:$P$13,Planejado!$B$5:$B$13,"Jurídico")</f>
         <v/>
       </c>
       <c r="C13" s="26">
-        <f>SUMIFS(Realizado!$P$5:$P$14,Realizado!$B$5:$B$14,"Jurídico")</f>
+        <f>SUMIFS(Realizado!$P$5:$P$13,Realizado!$B$5:$B$13,"Jurídico")</f>
         <v/>
       </c>
       <c r="D13" s="26">
@@ -4446,11 +4245,11 @@
         </is>
       </c>
       <c r="B14" s="43">
-        <f>SUMIFS(Planejado!$Q$5:$Q$14,Planejado!$B$5:$B$14,"Jurídico")</f>
+        <f>SUMIFS(Planejado!$Q$5:$Q$13,Planejado!$B$5:$B$13,"Jurídico")</f>
         <v/>
       </c>
       <c r="C14" s="43">
-        <f>SUMIFS(Realizado!$Q$5:$Q$14,Realizado!$B$5:$B$14,"Jurídico")</f>
+        <f>SUMIFS(Realizado!$Q$5:$Q$13,Realizado!$B$5:$B$13,"Jurídico")</f>
         <v/>
       </c>
       <c r="D14" s="43">
@@ -4481,11 +4280,11 @@
         </is>
       </c>
       <c r="B15" s="26">
-        <f>SUMIFS(Planejado!$R$5:$R$14,Planejado!$B$5:$B$14,"Jurídico")</f>
+        <f>SUMIFS(Planejado!$R$5:$R$13,Planejado!$B$5:$B$13,"Jurídico")</f>
         <v/>
       </c>
       <c r="C15" s="26">
-        <f>SUMIFS(Realizado!$R$5:$R$14,Realizado!$B$5:$B$14,"Jurídico")</f>
+        <f>SUMIFS(Realizado!$R$5:$R$13,Realizado!$B$5:$B$13,"Jurídico")</f>
         <v/>
       </c>
       <c r="D15" s="26">
@@ -4516,11 +4315,11 @@
         </is>
       </c>
       <c r="B16" s="43">
-        <f>SUMIFS(Planejado!$S$5:$S$14,Planejado!$B$5:$B$14,"Jurídico")</f>
+        <f>SUMIFS(Planejado!$S$5:$S$13,Planejado!$B$5:$B$13,"Jurídico")</f>
         <v/>
       </c>
       <c r="C16" s="43">
-        <f>SUMIFS(Realizado!$S$5:$S$14,Realizado!$B$5:$B$14,"Jurídico")</f>
+        <f>SUMIFS(Realizado!$S$5:$S$13,Realizado!$B$5:$B$13,"Jurídico")</f>
         <v/>
       </c>
       <c r="D16" s="43">
@@ -4597,7 +4396,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4673,11 +4472,11 @@
         </is>
       </c>
       <c r="B5" s="26">
-        <f>SUMIFS(Comparativo!$I$6:$I$15,Comparativo!$E$6:$E$15,$A5,Comparativo!$B$6:$B$15,"Jurídico")</f>
+        <f>SUMIFS(Comparativo!$I$6:$I$14,Comparativo!$E$6:$E$14,$A5,Comparativo!$B$6:$B$14,"Jurídico")</f>
         <v/>
       </c>
       <c r="C5" s="26">
-        <f>SUMIFS(Comparativo!$J$6:$J$15,Comparativo!$E$6:$E$15,$A5,Comparativo!$B$6:$B$15,"Jurídico")</f>
+        <f>SUMIFS(Comparativo!$J$6:$J$14,Comparativo!$E$6:$E$14,$A5,Comparativo!$B$6:$B$14,"Jurídico")</f>
         <v/>
       </c>
       <c r="D5" s="26">
@@ -4697,22 +4496,22 @@
         <v/>
       </c>
       <c r="H5" s="26">
-        <f>SUMIFS(Planejado!$T$5:$T$14,Planejado!$G$5:$G$14,$A5)</f>
+        <f>SUMIFS(Planejado!$T$5:$T$13,Planejado!$G$5:$G$13,$A5)</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="46" t="inlineStr">
         <is>
-          <t>Encargos e Benefícios - CLT</t>
+          <t>Pessoal - PJ</t>
         </is>
       </c>
       <c r="B6" s="43">
-        <f>SUMIFS(Comparativo!$I$6:$I$15,Comparativo!$E$6:$E$15,$A6,Comparativo!$B$6:$B$15,"Jurídico")</f>
+        <f>SUMIFS(Comparativo!$I$6:$I$14,Comparativo!$E$6:$E$14,$A6,Comparativo!$B$6:$B$14,"Jurídico")</f>
         <v/>
       </c>
       <c r="C6" s="43">
-        <f>SUMIFS(Comparativo!$J$6:$J$15,Comparativo!$E$6:$E$15,$A6,Comparativo!$B$6:$B$15,"Jurídico")</f>
+        <f>SUMIFS(Comparativo!$J$6:$J$14,Comparativo!$E$6:$E$14,$A6,Comparativo!$B$6:$B$14,"Jurídico")</f>
         <v/>
       </c>
       <c r="D6" s="43">
@@ -4732,22 +4531,22 @@
         <v/>
       </c>
       <c r="H6" s="43">
-        <f>SUMIFS(Planejado!$T$5:$T$14,Planejado!$G$5:$G$14,$A6)</f>
+        <f>SUMIFS(Planejado!$T$5:$T$13,Planejado!$G$5:$G$13,$A6)</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="44" t="inlineStr">
         <is>
-          <t>Pessoal - PJ</t>
+          <t>Licenças de Softwares</t>
         </is>
       </c>
       <c r="B7" s="26">
-        <f>SUMIFS(Comparativo!$I$6:$I$15,Comparativo!$E$6:$E$15,$A7,Comparativo!$B$6:$B$15,"Jurídico")</f>
+        <f>SUMIFS(Comparativo!$I$6:$I$14,Comparativo!$E$6:$E$14,$A7,Comparativo!$B$6:$B$14,"Jurídico")</f>
         <v/>
       </c>
       <c r="C7" s="26">
-        <f>SUMIFS(Comparativo!$J$6:$J$15,Comparativo!$E$6:$E$15,$A7,Comparativo!$B$6:$B$15,"Jurídico")</f>
+        <f>SUMIFS(Comparativo!$J$6:$J$14,Comparativo!$E$6:$E$14,$A7,Comparativo!$B$6:$B$14,"Jurídico")</f>
         <v/>
       </c>
       <c r="D7" s="26">
@@ -4767,22 +4566,22 @@
         <v/>
       </c>
       <c r="H7" s="26">
-        <f>SUMIFS(Planejado!$T$5:$T$14,Planejado!$G$5:$G$14,$A7)</f>
+        <f>SUMIFS(Planejado!$T$5:$T$13,Planejado!$G$5:$G$13,$A7)</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="46" t="inlineStr">
         <is>
-          <t>Licenças de Softwares</t>
+          <t>Custeio de Treinamento</t>
         </is>
       </c>
       <c r="B8" s="43">
-        <f>SUMIFS(Comparativo!$I$6:$I$15,Comparativo!$E$6:$E$15,$A8,Comparativo!$B$6:$B$15,"Jurídico")</f>
+        <f>SUMIFS(Comparativo!$I$6:$I$14,Comparativo!$E$6:$E$14,$A8,Comparativo!$B$6:$B$14,"Jurídico")</f>
         <v/>
       </c>
       <c r="C8" s="43">
-        <f>SUMIFS(Comparativo!$J$6:$J$15,Comparativo!$E$6:$E$15,$A8,Comparativo!$B$6:$B$15,"Jurídico")</f>
+        <f>SUMIFS(Comparativo!$J$6:$J$14,Comparativo!$E$6:$E$14,$A8,Comparativo!$B$6:$B$14,"Jurídico")</f>
         <v/>
       </c>
       <c r="D8" s="43">
@@ -4802,22 +4601,22 @@
         <v/>
       </c>
       <c r="H8" s="43">
-        <f>SUMIFS(Planejado!$T$5:$T$14,Planejado!$G$5:$G$14,$A8)</f>
+        <f>SUMIFS(Planejado!$T$5:$T$13,Planejado!$G$5:$G$13,$A8)</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="44" t="inlineStr">
         <is>
-          <t>Custeio de Treinamento</t>
+          <t>Prêmios</t>
         </is>
       </c>
       <c r="B9" s="26">
-        <f>SUMIFS(Comparativo!$I$6:$I$15,Comparativo!$E$6:$E$15,$A9,Comparativo!$B$6:$B$15,"Jurídico")</f>
+        <f>SUMIFS(Comparativo!$I$6:$I$14,Comparativo!$E$6:$E$14,$A9,Comparativo!$B$6:$B$14,"Jurídico")</f>
         <v/>
       </c>
       <c r="C9" s="26">
-        <f>SUMIFS(Comparativo!$J$6:$J$15,Comparativo!$E$6:$E$15,$A9,Comparativo!$B$6:$B$15,"Jurídico")</f>
+        <f>SUMIFS(Comparativo!$J$6:$J$14,Comparativo!$E$6:$E$14,$A9,Comparativo!$B$6:$B$14,"Jurídico")</f>
         <v/>
       </c>
       <c r="D9" s="26">
@@ -4837,77 +4636,42 @@
         <v/>
       </c>
       <c r="H9" s="26">
-        <f>SUMIFS(Planejado!$T$5:$T$14,Planejado!$G$5:$G$14,$A9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="46" t="inlineStr">
-        <is>
-          <t>Prêmios</t>
-        </is>
-      </c>
-      <c r="B10" s="43">
-        <f>SUMIFS(Comparativo!$I$6:$I$15,Comparativo!$E$6:$E$15,$A10,Comparativo!$B$6:$B$15,"Jurídico")</f>
-        <v/>
-      </c>
-      <c r="C10" s="43">
-        <f>SUMIFS(Comparativo!$J$6:$J$15,Comparativo!$E$6:$E$15,$A10,Comparativo!$B$6:$B$15,"Jurídico")</f>
-        <v/>
-      </c>
-      <c r="D10" s="43">
-        <f>B10</f>
-        <v/>
-      </c>
-      <c r="E10" s="43">
-        <f>C10</f>
-        <v/>
-      </c>
-      <c r="F10" s="43">
-        <f>E10-D10</f>
-        <v/>
-      </c>
-      <c r="G10" s="47">
+        <f>SUMIFS(Planejado!$T$5:$T$13,Planejado!$G$5:$G$13,$A9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B10" s="31">
+        <f>SUM(B5:B9)</f>
+        <v/>
+      </c>
+      <c r="C10" s="31">
+        <f>SUM(C5:C9)</f>
+        <v/>
+      </c>
+      <c r="D10" s="31">
+        <f>SUM(D5:D9)</f>
+        <v/>
+      </c>
+      <c r="E10" s="31">
+        <f>SUM(E5:E9)</f>
+        <v/>
+      </c>
+      <c r="F10" s="31">
+        <f>SUM(F5:F9)</f>
+        <v/>
+      </c>
+      <c r="G10" s="48">
         <f>IFERROR(F10/D10,"")</f>
         <v/>
       </c>
-      <c r="H10" s="43">
-        <f>SUMIFS(Planejado!$T$5:$T$14,Planejado!$G$5:$G$14,$A10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="30" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B11" s="31">
-        <f>SUM(B5:B10)</f>
-        <v/>
-      </c>
-      <c r="C11" s="31">
-        <f>SUM(C5:C10)</f>
-        <v/>
-      </c>
-      <c r="D11" s="31">
-        <f>SUM(D5:D10)</f>
-        <v/>
-      </c>
-      <c r="E11" s="31">
-        <f>SUM(E5:E10)</f>
-        <v/>
-      </c>
-      <c r="F11" s="31">
-        <f>SUM(F5:F10)</f>
-        <v/>
-      </c>
-      <c r="G11" s="48">
-        <f>IFERROR(F11/D11,"")</f>
-        <v/>
-      </c>
-      <c r="H11" s="31">
-        <f>SUM(H5:H10)</f>
+      <c r="H10" s="31">
+        <f>SUM(H5:H9)</f>
         <v/>
       </c>
     </row>
@@ -4916,7 +4680,7 @@
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F10">
+  <conditionalFormatting sqref="F5:F9">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -4999,17 +4763,17 @@
       </c>
       <c r="B5" s="50" t="inlineStr">
         <is>
-          <t>Encargos da Geovanna — CAMPO A PREENCHER</t>
+          <t>Custo total da Geovanna — A LANÇAR</t>
         </is>
       </c>
       <c r="C5" s="50" t="inlineStr">
         <is>
-          <t>A linha JUR-E02B recebe os encargos e benefícios sobre o salário bruto (INSS patronal, FGTS, provisões de 13º e férias, VT/VR, plano de saúde). Hoje está em branco.</t>
+          <t>O planejado dela é R$ 4.825,52/mês, que é o custo total orçado na ficha (salário + encargos de folha + benefícios). O dado disponível hoje é só o salário bruto, R$ 2.886,91/mês. O realizado está em branco.</t>
         </is>
       </c>
       <c r="D5" s="50" t="inlineStr">
         <is>
-          <t>Enquanto não for preenchida, a folha do Jurídico aparece R$ 1.938,61/mês abaixo do orçado — economia que não existe, é só encargo não lançado.</t>
+          <t>Lançar só o bruto contra um orçado de custo total mostraria economia de R$ 1.938,61/mês que não existe. Peça ao RH o custo total mensal dela, ou o bruto mais os encargos para somar antes de lançar.</t>
         </is>
       </c>
       <c r="E5" s="50" t="inlineStr">
@@ -5019,7 +4783,7 @@
       </c>
       <c r="F5" s="51" t="inlineStr">
         <is>
-          <t>PREENCHER</t>
+          <t>A LANÇAR</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(orcamento): realizado replicado de jan a jul
Gestora confirmou que os valores informados valem desde janeiro, nao so
a partir de maio. Os sete meses fechados passam a ter lancamento; ago a
dez ficam em branco e serao confirmados no decorrer do ano.

Jonathan lancado com zero em jan-mar por causa da entrada em abril
deduzida do total de 9 meses da ficha — ponto em aberto, ver abaixo.

Geovanna e Vinicius seguem sem lancamento: falta o custo total.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_JURIDICO_2026.xlsx
+++ b/orcamento/Orcamento_JURIDICO_2026.xlsx
@@ -3303,10 +3303,18 @@
         <f>Planejado!G5</f>
         <v/>
       </c>
-      <c r="H5" s="37" t="n"/>
-      <c r="I5" s="37" t="n"/>
-      <c r="J5" s="37" t="n"/>
-      <c r="K5" s="37" t="n"/>
+      <c r="H5" s="37" t="n">
+        <v>8818</v>
+      </c>
+      <c r="I5" s="37" t="n">
+        <v>8818</v>
+      </c>
+      <c r="J5" s="37" t="n">
+        <v>8818</v>
+      </c>
+      <c r="K5" s="37" t="n">
+        <v>8818</v>
+      </c>
       <c r="L5" s="37" t="n">
         <v>8818</v>
       </c>
@@ -3409,10 +3417,18 @@
         <f>Planejado!G7</f>
         <v/>
       </c>
-      <c r="H7" s="37" t="n"/>
-      <c r="I7" s="37" t="n"/>
-      <c r="J7" s="37" t="n"/>
-      <c r="K7" s="37" t="n"/>
+      <c r="H7" s="37" t="n">
+        <v>5500</v>
+      </c>
+      <c r="I7" s="37" t="n">
+        <v>5500</v>
+      </c>
+      <c r="J7" s="37" t="n">
+        <v>5500</v>
+      </c>
+      <c r="K7" s="37" t="n">
+        <v>5500</v>
+      </c>
       <c r="L7" s="37" t="n">
         <v>5500</v>
       </c>
@@ -3467,10 +3483,18 @@
         <f>Planejado!G8</f>
         <v/>
       </c>
-      <c r="H8" s="37" t="n"/>
-      <c r="I8" s="37" t="n"/>
-      <c r="J8" s="37" t="n"/>
-      <c r="K8" s="37" t="n"/>
+      <c r="H8" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="37" t="n">
+        <v>0</v>
+      </c>
       <c r="L8" s="37" t="n">
         <v>0</v>
       </c>
@@ -3525,10 +3549,18 @@
         <f>Planejado!G9</f>
         <v/>
       </c>
-      <c r="H9" s="37" t="n"/>
-      <c r="I9" s="37" t="n"/>
-      <c r="J9" s="37" t="n"/>
-      <c r="K9" s="37" t="n"/>
+      <c r="H9" s="37" t="n">
+        <v>136</v>
+      </c>
+      <c r="I9" s="37" t="n">
+        <v>136</v>
+      </c>
+      <c r="J9" s="37" t="n">
+        <v>136</v>
+      </c>
+      <c r="K9" s="37" t="n">
+        <v>136</v>
+      </c>
       <c r="L9" s="37" t="n">
         <v>136</v>
       </c>
@@ -3583,10 +3615,18 @@
         <f>Planejado!G10</f>
         <v/>
       </c>
-      <c r="H10" s="37" t="n"/>
-      <c r="I10" s="37" t="n"/>
-      <c r="J10" s="37" t="n"/>
-      <c r="K10" s="37" t="n"/>
+      <c r="H10" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="37" t="n">
+        <v>0</v>
+      </c>
       <c r="L10" s="37" t="n">
         <v>0</v>
       </c>
@@ -3641,10 +3681,18 @@
         <f>Planejado!G11</f>
         <v/>
       </c>
-      <c r="H11" s="37" t="n"/>
-      <c r="I11" s="37" t="n"/>
-      <c r="J11" s="37" t="n"/>
-      <c r="K11" s="37" t="n"/>
+      <c r="H11" s="37" t="n">
+        <v>970</v>
+      </c>
+      <c r="I11" s="37" t="n">
+        <v>970</v>
+      </c>
+      <c r="J11" s="37" t="n">
+        <v>970</v>
+      </c>
+      <c r="K11" s="37" t="n">
+        <v>970</v>
+      </c>
       <c r="L11" s="37" t="n">
         <v>970</v>
       </c>
@@ -3695,10 +3743,18 @@
         <f>Planejado!G12</f>
         <v/>
       </c>
-      <c r="H12" s="37" t="n"/>
-      <c r="I12" s="37" t="n"/>
-      <c r="J12" s="37" t="n"/>
-      <c r="K12" s="37" t="n"/>
+      <c r="H12" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="37" t="n">
+        <v>0</v>
+      </c>
       <c r="L12" s="37" t="n">
         <v>0</v>
       </c>
@@ -3753,22 +3809,40 @@
         <f>Planejado!G13</f>
         <v/>
       </c>
-      <c r="H13" s="37" t="n"/>
-      <c r="I13" s="37" t="n"/>
-      <c r="J13" s="37" t="n"/>
-      <c r="K13" s="37" t="n"/>
-      <c r="L13" s="37" t="n"/>
-      <c r="M13" s="37" t="n"/>
-      <c r="N13" s="37" t="n"/>
+      <c r="H13" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="37" t="n">
+        <v>0</v>
+      </c>
       <c r="O13" s="37" t="n"/>
       <c r="T13" s="33">
         <f>SUM(H13:S13)</f>
         <v/>
       </c>
-      <c r="U13" s="38" t="n"/>
+      <c r="U13" s="38" t="inlineStr">
+        <is>
+          <t>Gestora, 05/08/26</t>
+        </is>
+      </c>
       <c r="V13" s="38" t="inlineStr">
         <is>
-          <t>Bonificação de ago/26 a confirmar</t>
+          <t>Sem parcela no 1º semestre; bonificação de ago/26 a confirmar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(orcamento): planejado da Thamar revisado a partir de agosto
Gestora confirmou que ela recebe R$ 5.500 desde jan/26, nao desde maio.
A revisao do planejado, que estava comecando em out, passa para ago —
o primeiro mes ainda nao realizado. Os sete meses fechados ficam no
baseline de R$ 5.000 para o desvio de R$ 3.500 continuar visivel.

Confirmada tambem a entrada do Jonathan em abril, ja lancada.

Juridico: R$ 291.730,42. Geral: R$ 548.548,72.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_JURIDICO_2026.xlsx
+++ b/orcamento/Orcamento_JURIDICO_2026.xlsx
@@ -2560,7 +2560,7 @@
       </c>
       <c r="E7" s="25" t="inlineStr">
         <is>
-          <t>Advogada — reajuste permanente de R$ 5.000 para R$ 5.500 (revisado a partir de out/26)</t>
+          <t>Advogada — recebe R$ 5.500/mês desde jan/26 contra R$ 5.000 orçados. Planejado revisado para R$ 5.500 a partir de ago/26</t>
         </is>
       </c>
       <c r="F7" s="24" t="inlineStr">
@@ -2595,10 +2595,10 @@
         <v>5000</v>
       </c>
       <c r="O7" s="26" t="n">
-        <v>5000</v>
+        <v>5500</v>
       </c>
       <c r="P7" s="26" t="n">
-        <v>5000</v>
+        <v>5500</v>
       </c>
       <c r="Q7" s="26" t="n">
         <v>5500</v>
@@ -4869,17 +4869,17 @@
       </c>
       <c r="B6" s="53" t="inlineStr">
         <is>
-          <t>Reajuste da Thamar — revisão orçamentária</t>
+          <t>Thamar acima do orçado desde janeiro</t>
         </is>
       </c>
       <c r="C6" s="53" t="inlineStr">
         <is>
-          <t>Reajuste permanente de R$ 5.000 para R$ 5.500/mês, em vigor desde mai/26. O planejado foi mantido em R$ 5.000 nos meses já realizados (para o desvio ficar visível) e revisado para R$ 5.500 de out a dez.</t>
+          <t>Recebe R$ 5.500/mês desde jan/26 contra R$ 5.000 orçados. O planejado foi mantido em R$ 5.000 nos sete meses fechados (para o desvio ficar visível) e revisado para R$ 5.500 de ago a dez.</t>
         </is>
       </c>
       <c r="D6" s="53" t="inlineStr">
         <is>
-          <t>Desvio já incorrido de R$ 500/mês. Ao contrário do aumento do Vinicius, este estourou o orçado: não havia folga na linha dela.</t>
+          <t>R$ 3.500 já gastos acima do orçado em jan–jul, e mais R$ 2.500 previstos até dezembro. Ao contrário do aumento do Vinicius, este estourou o orçado: não havia folga na linha dela. Orçamento do Jurídico sobe para R$ 291.730,42.</t>
         </is>
       </c>
       <c r="E6" s="53" t="inlineStr">

</xml_diff>

<commit_message>
fix(orcamento): historico salarial da Thamar em jan-fev
Recebia R$ 4.500/mes em jan e fev e teve aumento de R$ 1.000 em mar/26,
passando a R$ 5.500. Antes o realizado dela estava lancado como R$ 5.500
o ano todo.

Efeito no acumulado jan-jul: o desvio cai de R$ 3.500 para R$ 1.500,
resultado de -R$ 1.000 em jan-fev (abaixo do orcado) e +R$ 2.500 em
mar-jul (acima). O planejado segue no baseline de R$ 5.000 nos meses
fechados e revisado para R$ 5.500 de ago em diante.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_JURIDICO_2026.xlsx
+++ b/orcamento/Orcamento_JURIDICO_2026.xlsx
@@ -2560,7 +2560,7 @@
       </c>
       <c r="E7" s="25" t="inlineStr">
         <is>
-          <t>Advogada — recebe R$ 5.500/mês desde jan/26 contra R$ 5.000 orçados. Planejado revisado para R$ 5.500 a partir de ago/26</t>
+          <t>Advogada — recebia R$ 4.500/mês em jan–fev e passou a R$ 5.500 em mar/26 (aumento de R$ 1.000), contra R$ 5.000 orçados. Planejado revisado para R$ 5.500 a partir de ago/26</t>
         </is>
       </c>
       <c r="F7" s="24" t="inlineStr">
@@ -3418,10 +3418,10 @@
         <v/>
       </c>
       <c r="H7" s="37" t="n">
-        <v>5500</v>
+        <v>4500</v>
       </c>
       <c r="I7" s="37" t="n">
-        <v>5500</v>
+        <v>4500</v>
       </c>
       <c r="J7" s="37" t="n">
         <v>5500</v>
@@ -3450,7 +3450,7 @@
       </c>
       <c r="V7" s="38" t="inlineStr">
         <is>
-          <t>Reajuste permanente aplicado desde mai/26</t>
+          <t>R$ 4.500/mês em jan–fev; aumento de R$ 1.000 a partir de mar/26</t>
         </is>
       </c>
     </row>
@@ -4869,17 +4869,17 @@
       </c>
       <c r="B6" s="53" t="inlineStr">
         <is>
-          <t>Thamar acima do orçado desde janeiro</t>
+          <t>Aumento da Thamar em mar/26</t>
         </is>
       </c>
       <c r="C6" s="53" t="inlineStr">
         <is>
-          <t>Recebe R$ 5.500/mês desde jan/26 contra R$ 5.000 orçados. O planejado foi mantido em R$ 5.000 nos sete meses fechados (para o desvio ficar visível) e revisado para R$ 5.500 de ago a dez.</t>
+          <t>Recebia R$ 4.500/mês em jan e fev, abaixo dos R$ 5.000 orçados. Em mar/26 teve aumento de R$ 1.000 e passou a R$ 5.500, acima do orçado. O planejado foi mantido em R$ 5.000 nos sete meses fechados (para o desvio ficar visível) e revisado para R$ 5.500 de ago a dez.</t>
         </is>
       </c>
       <c r="D6" s="53" t="inlineStr">
         <is>
-          <t>R$ 3.500 já gastos acima do orçado em jan–jul, e mais R$ 2.500 previstos até dezembro. Ao contrário do aumento do Vinicius, este estourou o orçado: não havia folga na linha dela. Orçamento do Jurídico sobe para R$ 291.730,42.</t>
+          <t>No acumulado jan–jul o efeito líquido é de R$ 1.500 acima do orçado (−R$ 1.000 em jan–fev, +R$ 2.500 em mar–jul), e mais R$ 2.500 previstos até dezembro. Ao contrário do aumento do Vinicius, este estourou o orçado: não havia folga na linha dela.</t>
         </is>
       </c>
       <c r="E6" s="53" t="inlineStr">

</xml_diff>

<commit_message>
fix(orcamento): aumento da Thamar passa de mar para abr/26
Correcao da gestora. R$ 4.500/mes de jan a mar e R$ 5.500 de abr em
diante.

O desvio acumulado jan-jul cai de R$ 1.500 para R$ 500: sao -R$ 1.500
em jan-mar (abaixo do orcado) contra +R$ 2.000 em abr-jul (acima).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_JURIDICO_2026.xlsx
+++ b/orcamento/Orcamento_JURIDICO_2026.xlsx
@@ -2560,7 +2560,7 @@
       </c>
       <c r="E7" s="25" t="inlineStr">
         <is>
-          <t>Advogada — recebia R$ 4.500/mês em jan–fev e passou a R$ 5.500 em mar/26 (aumento de R$ 1.000), contra R$ 5.000 orçados. Planejado revisado para R$ 5.500 a partir de ago/26</t>
+          <t>Advogada — recebia R$ 4.500/mês em jan–mar e passou a R$ 5.500 em abr/26 (aumento de R$ 1.000), contra R$ 5.000 orçados. Planejado revisado para R$ 5.500 a partir de ago/26</t>
         </is>
       </c>
       <c r="F7" s="24" t="inlineStr">
@@ -3424,7 +3424,7 @@
         <v>4500</v>
       </c>
       <c r="J7" s="37" t="n">
-        <v>5500</v>
+        <v>4500</v>
       </c>
       <c r="K7" s="37" t="n">
         <v>5500</v>
@@ -3450,7 +3450,7 @@
       </c>
       <c r="V7" s="38" t="inlineStr">
         <is>
-          <t>R$ 4.500/mês em jan–fev; aumento de R$ 1.000 a partir de mar/26</t>
+          <t>R$ 4.500/mês em jan–mar; aumento de R$ 1.000 a partir de abr/26</t>
         </is>
       </c>
     </row>
@@ -4869,17 +4869,17 @@
       </c>
       <c r="B6" s="53" t="inlineStr">
         <is>
-          <t>Aumento da Thamar em mar/26</t>
+          <t>Aumento da Thamar em abr/26</t>
         </is>
       </c>
       <c r="C6" s="53" t="inlineStr">
         <is>
-          <t>Recebia R$ 4.500/mês em jan e fev, abaixo dos R$ 5.000 orçados. Em mar/26 teve aumento de R$ 1.000 e passou a R$ 5.500, acima do orçado. O planejado foi mantido em R$ 5.000 nos sete meses fechados (para o desvio ficar visível) e revisado para R$ 5.500 de ago a dez.</t>
+          <t>Recebia R$ 4.500/mês de jan a mar, abaixo dos R$ 5.000 orçados. Em abr/26 teve aumento de R$ 1.000 e passou a R$ 5.500, acima do orçado. O planejado foi mantido em R$ 5.000 nos sete meses fechados (para o desvio ficar visível) e revisado para R$ 5.500 de ago a dez.</t>
         </is>
       </c>
       <c r="D6" s="53" t="inlineStr">
         <is>
-          <t>No acumulado jan–jul o efeito líquido é de R$ 1.500 acima do orçado (−R$ 1.000 em jan–fev, +R$ 2.500 em mar–jul), e mais R$ 2.500 previstos até dezembro. Ao contrário do aumento do Vinicius, este estourou o orçado: não havia folga na linha dela.</t>
+          <t>No acumulado jan–jul o efeito líquido é de apenas R$ 500 acima do orçado (−R$ 1.500 em jan–mar, +R$ 2.000 em abr–jul), e mais R$ 2.500 previstos até dezembro. Ao contrário do aumento do Vinicius, este estourou o orçado: não havia folga na linha dela.</t>
         </is>
       </c>
       <c r="E6" s="53" t="inlineStr">

</xml_diff>

<commit_message>
fix(orcamento): valores reais do Miguel e defasagem caixa x competencia
Gestora informou R$ 6.750/mes de jan a jul, e R$ 8.818 pagos em 01/08
referentes a julho. Antes o realizado dele estava lancado como R$ 8.818
o ano todo.

A economia do Miguel no acumulado jan-jul passa de R$ 8.274 para
R$ 22.750, e a economia liquida do Juridico de R$ 16.460,79 para
R$ 30.936,79 (25% do orcado comparavel, projecao de R$ 53.034,50).

O detalhe do pagamento de 01/08 confirma que ha defasagem entre
prestacao e pagamento. Todo o realizado esta lancado por caixa, que e
como os valores foram informados; a pendencia de competencia x caixa
deixou de ser teorica e foi reescrita com a consequencia concreta — o
lancamento de jan/26 pode referir-se a dez/2025.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_JURIDICO_2026.xlsx
+++ b/orcamento/Orcamento_JURIDICO_2026.xlsx
@@ -3838,27 +3838,29 @@
         <v/>
       </c>
       <c r="H5" s="50" t="n">
+        <v>6750</v>
+      </c>
+      <c r="I5" s="50" t="n">
+        <v>6750</v>
+      </c>
+      <c r="J5" s="50" t="n">
+        <v>6750</v>
+      </c>
+      <c r="K5" s="50" t="n">
+        <v>6750</v>
+      </c>
+      <c r="L5" s="50" t="n">
+        <v>6750</v>
+      </c>
+      <c r="M5" s="50" t="n">
+        <v>6750</v>
+      </c>
+      <c r="N5" s="50" t="n">
+        <v>6750</v>
+      </c>
+      <c r="O5" s="50" t="n">
         <v>8818</v>
       </c>
-      <c r="I5" s="50" t="n">
-        <v>8818</v>
-      </c>
-      <c r="J5" s="50" t="n">
-        <v>8818</v>
-      </c>
-      <c r="K5" s="50" t="n">
-        <v>8818</v>
-      </c>
-      <c r="L5" s="50" t="n">
-        <v>8818</v>
-      </c>
-      <c r="M5" s="50" t="n">
-        <v>8818</v>
-      </c>
-      <c r="N5" s="50" t="n">
-        <v>8818</v>
-      </c>
-      <c r="O5" s="50" t="n"/>
       <c r="T5" s="46">
         <f>SUM(H5:S5)</f>
         <v/>
@@ -3870,7 +3872,7 @@
       </c>
       <c r="V5" s="51" t="inlineStr">
         <is>
-          <t>Valor cheio da nota — R$ 1.182/mês abaixo do contratado</t>
+          <t>R$ 6.750/mês de jan a jul; R$ 8.818 pagos em 01/08 (ref. julho). Lançado por caixa</t>
         </is>
       </c>
     </row>
@@ -5645,17 +5647,17 @@
       </c>
       <c r="B13" s="63" t="inlineStr">
         <is>
-          <t>Critério de competência x caixa</t>
+          <t>Competência x caixa — DEFASAGEM CONFIRMADA</t>
         </is>
       </c>
       <c r="C13" s="63" t="inlineStr">
         <is>
-          <t>Definir se o realizado será lançado pela data de pagamento (caixa) ou pelo mês de referência da despesa (competência).</t>
+          <t>O pagamento do Miguel de 01/08/26 refere-se a julho, então há pelo menos um prestador cujo pagamento cai no mês seguinte ao da prestação. Todo o realizado está lançado por CAIXA (mês em que o pagamento saiu), que é como os valores foram informados.</t>
         </is>
       </c>
       <c r="D13" s="63" t="inlineStr">
         <is>
-          <t>Misturar os dois critérios gera desvio artificial em meses de virada, principalmente em folha e prêmios.</t>
+          <t>Consequência: o valor lançado em jan/26 pode ser referente a dez/2025, e o serviço de dez/26 só aparecerá em jan/2027 — o ano fecha com 12 pagamentos, mas defasados em relação ao orçamento, que é de competência. Vale conferir quais contratos pagam no mês seguinte e decidir se o comparativo passa para competência.</t>
         </is>
       </c>
       <c r="E13" s="63" t="inlineStr">
@@ -5663,9 +5665,9 @@
           <t>Cristiane + Financeiro</t>
         </is>
       </c>
-      <c r="F13" s="68" t="inlineStr">
-        <is>
-          <t>EM ABERTO</t>
+      <c r="F13" s="69" t="inlineStr">
+        <is>
+          <t>DECIDIR</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(orcamento): Dra. Michele orcada em R$ 2.750/mes desde jan/26
Mao de obra que ficou de fora da ficha por esquecimento na montagem do
orcamento. Passa a ter planejado e realizado de R$ 2.750/mes pelo ano
inteiro, conforme a gestora.

Orcamento do Juridico sobe R$ 33.000, para R$ 324.730,42. Com planejado
igual ao realizado, a linha sai do ranking de estouros e fica "Dentro
do orcado" — o Astrea volta a ser o maior desvio da area.

Registrada divergencia a conferir no SIENGE: no extrato de contas
pagas, o unico lancamento isolado de R$ 2.750 e o de jul/26; de jan a
jun aparecem so honorarios por processo, que sao repasse. Ou os
pagamentos do fixo do 1o semestre sairam por outro centro de custo, ou
estao embutidos naqueles lancamentos.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_JURIDICO_2026.xlsx
+++ b/orcamento/Orcamento_JURIDICO_2026.xlsx
@@ -16144,7 +16144,7 @@
       </c>
       <c r="E8" s="37" t="inlineStr">
         <is>
-          <t>Advogada — NÃO CONSTAVA NA FICHA. R$ 2.750/mês fixos desde jul/26. Planejado a definir com a diretoria</t>
+          <t>Advogada — R$ 2.750/mês fixos desde jan/26. Não constava na ficha por esquecimento na montagem do orçamento; incluída na revisão</t>
         </is>
       </c>
       <c r="F8" s="36" t="inlineStr">
@@ -16158,40 +16158,40 @@
         </is>
       </c>
       <c r="H8" s="38" t="n">
-        <v>0</v>
+        <v>2750</v>
       </c>
       <c r="I8" s="38" t="n">
-        <v>0</v>
+        <v>2750</v>
       </c>
       <c r="J8" s="38" t="n">
-        <v>0</v>
+        <v>2750</v>
       </c>
       <c r="K8" s="38" t="n">
-        <v>0</v>
+        <v>2750</v>
       </c>
       <c r="L8" s="38" t="n">
-        <v>0</v>
+        <v>2750</v>
       </c>
       <c r="M8" s="38" t="n">
-        <v>0</v>
+        <v>2750</v>
       </c>
       <c r="N8" s="38" t="n">
-        <v>0</v>
+        <v>2750</v>
       </c>
       <c r="O8" s="38" t="n">
-        <v>0</v>
+        <v>2750</v>
       </c>
       <c r="P8" s="38" t="n">
-        <v>0</v>
+        <v>2750</v>
       </c>
       <c r="Q8" s="38" t="n">
-        <v>0</v>
+        <v>2750</v>
       </c>
       <c r="R8" s="38" t="n">
-        <v>0</v>
+        <v>2750</v>
       </c>
       <c r="S8" s="38" t="n">
-        <v>0</v>
+        <v>2750</v>
       </c>
       <c r="T8" s="46">
         <f>SUM(H8:S8)</f>
@@ -17104,22 +17104,22 @@
         <v/>
       </c>
       <c r="H8" s="50" t="n">
-        <v>0</v>
+        <v>2750</v>
       </c>
       <c r="I8" s="50" t="n">
-        <v>0</v>
+        <v>2750</v>
       </c>
       <c r="J8" s="50" t="n">
-        <v>0</v>
+        <v>2750</v>
       </c>
       <c r="K8" s="50" t="n">
-        <v>0</v>
+        <v>2750</v>
       </c>
       <c r="L8" s="50" t="n">
-        <v>0</v>
+        <v>2750</v>
       </c>
       <c r="M8" s="50" t="n">
-        <v>0</v>
+        <v>2750</v>
       </c>
       <c r="N8" s="50" t="n">
         <v>2750</v>
@@ -17135,12 +17135,12 @@
       </c>
       <c r="U8" s="51" t="inlineStr">
         <is>
-          <t>Extrato do financeiro</t>
+          <t>Gestora, 05/08/26</t>
         </is>
       </c>
       <c r="V8" s="51" t="inlineStr">
         <is>
-          <t>R$ 2.750/mês fixos a partir de jul/26. Os demais lançamentos em nome dela no extrato são REPASSE de honorários pagos pelo cliente — não são custo do departamento</t>
+          <t>R$ 2.750/mês fixos desde jan/26. Os demais lançamentos em nome dela no extrato são REPASSE de honorários pagos pelo cliente — não são custo do departamento</t>
         </is>
       </c>
     </row>
@@ -18891,27 +18891,27 @@
       </c>
       <c r="B15" s="63" t="inlineStr">
         <is>
-          <t>Dra. Michele fora do orçamento — INCLUIR</t>
+          <t>Dra. Michele incluída no orçamento</t>
         </is>
       </c>
       <c r="C15" s="63" t="inlineStr">
         <is>
-          <t>Advogada que presta serviço ao departamento e não foi incluída na ficha. Recebe R$ 2.750/mês fixos desde jul/26. A linha foi criada com planejado zerado, à espera da definição.</t>
+          <t>Mão de obra que ficou de fora da ficha por esquecimento na montagem do orçamento. Orçada em R$ 2.750/mês pelo ano inteiro, valor fixo em vigor desde jan/26.</t>
         </is>
       </c>
       <c r="D15" s="63" t="inlineStr">
         <is>
-          <t>A R$ 2.750/mês são R$ 33.000/ano, que hoje não têm previsão. Enquanto o planejado for zero, a linha aparece como 'Não orçado' e o valor entra inteiro como estouro. Definir o valor a orçar e a partir de quando.</t>
+          <t>Acréscimo de R$ 33.000 ao orçamento do Jurídico, que passa a R$ 324.730,42. CONFERIR NO SIENGE: no extrato de contas pagas, o único lançamento isolado de R$ 2.750 é o de jul/26 — de jan a jun aparecem apenas honorários por processo, que são repasse (item P). Ou os pagamentos do fixo de jan a jun saíram por outro centro de custo, ou estão embutidos naqueles lançamentos. Vale localizar antes da reunião. A justificativa da inclusão é pauta.</t>
         </is>
       </c>
       <c r="E15" s="63" t="inlineStr">
         <is>
-          <t>Cristiane + Diretoria</t>
-        </is>
-      </c>
-      <c r="F15" s="69" t="inlineStr">
-        <is>
-          <t>PAUTA REUNIÃO</t>
+          <t>Cristiane + Financeiro</t>
+        </is>
+      </c>
+      <c r="F15" s="70" t="inlineStr">
+        <is>
+          <t>CONFERIR</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(orcamento): divergencia da Dra. Michele explicada
Nao havia pagamento faltando: de jan a jun o fixo de R$ 2.750 vem
somado aos honorarios de repasse no mesmo credor, e a soma bate em
cinco dos seis meses. Jun/26 fica abaixo do fixo porque o pagamento
caiu em jul — e o lancamento isolado de R$ 2.750 que aparece la.

Item O passa de CONFERIR para APLICADO.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_JURIDICO_2026.xlsx
+++ b/orcamento/Orcamento_JURIDICO_2026.xlsx
@@ -18901,17 +18901,17 @@
       </c>
       <c r="D15" s="63" t="inlineStr">
         <is>
-          <t>Acréscimo de R$ 33.000 ao orçamento do Jurídico, que passa a R$ 324.730,42. CONFERIR NO SIENGE: no extrato de contas pagas, o único lançamento isolado de R$ 2.750 é o de jul/26 — de jan a jun aparecem apenas honorários por processo, que são repasse (item P). Ou os pagamentos do fixo de jan a jun saíram por outro centro de custo, ou estão embutidos naqueles lançamentos. Vale localizar antes da reunião. A justificativa da inclusão é pauta.</t>
+          <t>Acréscimo de R$ 33.000 ao orçamento do Jurídico, que passa a R$ 324.730,42. No extrato, o fixo de jan a jun vem somado aos honorários de repasse no mesmo credor: o total mensal (R$ 3.739 a R$ 4.326) é o fixo de R$ 2.750 mais o repasse, que o cliente paga e a empresa apenas transfere. Só jun/26 fica abaixo do fixo (R$ 1.036,92), provavelmente porque o pagamento daquele mês caiu em jul — é o lançamento isolado de R$ 2.750 que aparece lá. A justificativa da inclusão é pauta da reunião.</t>
         </is>
       </c>
       <c r="E15" s="63" t="inlineStr">
         <is>
-          <t>Cristiane + Financeiro</t>
-        </is>
-      </c>
-      <c r="F15" s="70" t="inlineStr">
-        <is>
-          <t>CONFERIR</t>
+          <t>Cristiane + Diretoria</t>
+        </is>
+      </c>
+      <c r="F15" s="67" t="inlineStr">
+        <is>
+          <t>APLICADO</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(orcamento): defasagem dos PJs nomeada por area e alerta no Jonathan
Gestora confirmou que os PJs do TI recebem no mes seguinte como os do
Juridico. A pendencia 7 passa a nomear os afetados: Miguel, Thamar e
Dra. Michele no Juridico; Elias e Jonathan no TI.

Registrado um descasamento especifico no Jonathan: o planejado comeca
em abr/26 por competencia e o realizado tambem foi lancado a partir de
abr por caixa. Se ele recebe no mes seguinte, o pagamento de abril e
servico de marco — ou a entrada foi em marco, ou o realizado de abril
deveria ser zero.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_JURIDICO_2026.xlsx
+++ b/orcamento/Orcamento_JURIDICO_2026.xlsx
@@ -20341,12 +20341,12 @@
       </c>
       <c r="C18" s="66" t="inlineStr">
         <is>
-          <t>Confirmado pela gestora: TODOS os PJs prestam o serviço e recebem no mês seguinte. O que foi pago em jan/26 é serviço de dez/2025, e o serviço de dez/26 só será pago em jan/2027. Hoje o realizado está lançado por CAIXA (mês do pagamento), que é como os valores foram informados, enquanto o orçamento foi montado por COMPETÊNCIA (mês do serviço). São bases diferentes no mesmo comparativo.</t>
+          <t>Confirmado pela gestora: TODOS os PJs das duas áreas prestam o serviço e recebem no mês seguinte — no Jurídico, Miguel, Thamar e Dra. Michele; no TI, Elias e Jonathan. O que foi pago em jan/26 é serviço de dez/2025, e o serviço de dez/26 só será pago em jan/2027. Hoje o realizado está lançado por CAIXA (mês do pagamento), que é como os valores foram informados, enquanto o orçamento foi montado por COMPETÊNCIA (mês do serviço). São bases diferentes no mesmo comparativo.</t>
         </is>
       </c>
       <c r="D18" s="66" t="inlineStr">
         <is>
-          <t>RECOMENDAÇÃO: migrar para competência, deslocando os PJs um mês para trás. Motivos: (1) o orçamento já é de competência, então acaba a comparação de bases diferentes; (2) por caixa, o ano de 2026 carrega um mês de 2025 e perde dez/26, o que distorce sempre que o valor muda no meio do ano — no Miguel, R$ 47.250 por caixa contra R$ 49.318 por competência em jan–jul, R$ 2.068 de diferença; (3) o SIENGE gera os dois regimes, então é escolha de configuração. Contra: caixa é mais fácil de bater com o extrato bancário. Decidir UMA vez e manter, senão o histórico mistura critérios.</t>
+          <t>RECOMENDAÇÃO: migrar para competência, deslocando os PJs um mês para trás. Motivos: (1) o orçamento já é de competência, então acaba a comparação de bases diferentes; (2) por caixa, o ano de 2026 carrega um mês de 2025 e perde dez/26, o que distorce sempre que o valor muda no meio do ano — no Miguel, R$ 47.250 por caixa contra R$ 49.318 por competência em jan–jul, R$ 2.068 de diferença; (3) o SIENGE gera os dois regimes, então é escolha de configuração. Contra: caixa é mais fácil de bater com o extrato bancário. Decidir UMA vez e manter, senão o histórico mistura critérios. ATENÇÃO NO JONATHAN: o planejado dele começa em abr/26 (competência) e o realizado também foi lançado a partir de abr (caixa) — se ele recebe no mês seguinte, o pagamento de abril é serviço de março, e ou a entrada dele foi em março, ou o realizado de abril deveria ser zero. Conferir junto com a decisão do regime.</t>
         </is>
       </c>
       <c r="E18" s="66" t="inlineStr">

</xml_diff>

<commit_message>
feat(orcamento): pendencia de reclassificacao do Adapta
Os pagamentos do Adapta (contrato 4134643529) estao no centro de custo
Juridico no SIENGE: R$ 575/mes de jan a mai e R$ 476 em jun, R$ 3.351
no total. Nao e despesa do Juridico — e ferramenta de IA de uso
transversal, e a gestora confirmou o erro de classificacao.

Nova pendencia Q, visivel nas duas planilhas: enquanto nao for
corrigido, o Juridico carrega R$ 3.351 que nao sao dele e o TI aparece
sem um gasto que e seu. A abertura do novo centro de custo e a
oportunidade de acertar a classificacao na origem.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_JURIDICO_2026.xlsx
+++ b/orcamento/Orcamento_JURIDICO_2026.xlsx
@@ -19855,7 +19855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -20267,22 +20267,22 @@
     <row r="16" ht="58" customHeight="1">
       <c r="A16" s="65" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="B16" s="66" t="inlineStr">
         <is>
-          <t>Extrato contém REPASSES, não só custo</t>
+          <t>Adapta lançado no centro de custo errado — RECLASSIFICAR</t>
         </is>
       </c>
       <c r="C16" s="66" t="inlineStr">
         <is>
-          <t>Os lançamentos em nome da Dra. Michele até jun/26 (R$ 20.821,53) são repasse: o cliente paga à empresa e a empresa repassa a ela. Não são custo do departamento e por isso não foram lançados no realizado.</t>
+          <t>Os pagamentos do Adapta (ADAPTA EDUCACAO LTDA, contrato 4134643529) estão no centro de custo Jurídico no SIENGE: R$ 575,00/mês de jan a mai e R$ 476,00 em jun, todos com vencimento dia 15. Total de R$ 3.351,00 em seis meses. Não é despesa do Jurídico — é ferramenta de IA, de uso transversal.</t>
         </is>
       </c>
       <c r="D16" s="66" t="inlineStr">
         <is>
-          <t>Vale a mesma checagem nos outros credores das abas 'Contas Pagas' antes de usá-los como custo — em especial custas processuais e honorários de terceiros, que podem ser reembolsados pelo cliente. O total de R$ 446.577,92 do centro de custo Jurídico no extrato NÃO é despesa líquida do departamento.</t>
+          <t>Reclassificar no SIENGE para o centro de custo correto e aplicar o rateio do item L. Enquanto não for corrigido, o Jurídico carrega R$ 3.351 que não são dele e o TI aparece sem um gasto que é seu — as duas áreas ficam com o comparativo errado. Aproveitar a abertura do novo centro de custo para acertar a classificação desde a origem.</t>
         </is>
       </c>
       <c r="E16" s="66" t="inlineStr">
@@ -20290,71 +20290,103 @@
           <t>Cristiane + Financeiro</t>
         </is>
       </c>
-      <c r="F16" s="70" t="inlineStr">
-        <is>
-          <t>CONFERIR</t>
+      <c r="F16" s="64" t="inlineStr">
+        <is>
+          <t>RECLASSIFICAR</t>
         </is>
       </c>
     </row>
     <row r="17" ht="58" customHeight="1">
       <c r="A17" s="62" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B17" s="63" t="inlineStr">
         <is>
-          <t>ORÇAMENTO VEIO ERRADO — Astrea e Jusbrasil</t>
+          <t>Extrato contém REPASSES, não só custo</t>
         </is>
       </c>
       <c r="C17" s="63" t="inlineStr">
         <is>
-          <t>ASTREA: orçado R$ 112,07/mês, o que dá R$ 1.344,84 no ano — praticamente o valor de UMA das cinco parcelas (R$ 1.346,28). Quem montou a ficha tomou uma parcela pelo custo total do ano. O custo real da anuidade foi R$ 6.731,40, 5x o orçado. JUSBRASIL: orçado R$ 104,90/mês contra R$ 136,00 reais (1,3x), R$ 373,20 no ano. PAUTA PARA A REUNIÃO COM A DIRETORIA.</t>
+          <t>Os lançamentos em nome da Dra. Michele até jun/26 (R$ 20.821,53) são repasse: o cliente paga à empresa e a empresa repassa a ela. Não são custo do departamento e por isso não foram lançados no realizado.</t>
         </is>
       </c>
       <c r="D17" s="63" t="inlineStr">
         <is>
-          <t>Subdimensionamento de R$ 5.759,76 no ano (R$ 5.386,56 do Astrea + R$ 373,20 do Jusbrasil). O planejado das duas linhas foi mantido como veio na ficha, de propósito, para o erro aparecer no comparativo em vez de ser corrigido em silêncio. Não é estouro de gestão: é erro na origem. Como o Astrea será cancelado, o efeito prático é só de 2026 — mas o método de orçar serviços parcelados precisa ser revisto para o ano que vem.</t>
+          <t>Vale a mesma checagem nos outros credores das abas 'Contas Pagas' antes de usá-los como custo — em especial custas processuais e honorários de terceiros, que podem ser reembolsados pelo cliente. O total de R$ 446.577,92 do centro de custo Jurídico no extrato NÃO é despesa líquida do departamento.</t>
         </is>
       </c>
       <c r="E17" s="63" t="inlineStr">
         <is>
-          <t>Cristiane + Diretoria</t>
-        </is>
-      </c>
-      <c r="F17" s="69" t="inlineStr">
-        <is>
-          <t>PAUTA REUNIÃO</t>
+          <t>Cristiane + Financeiro</t>
+        </is>
+      </c>
+      <c r="F17" s="70" t="inlineStr">
+        <is>
+          <t>CONFERIR</t>
         </is>
       </c>
     </row>
     <row r="18" ht="58" customHeight="1">
       <c r="A18" s="65" t="inlineStr">
         <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="B18" s="66" t="inlineStr">
+        <is>
+          <t>ORÇAMENTO VEIO ERRADO — Astrea e Jusbrasil</t>
+        </is>
+      </c>
+      <c r="C18" s="66" t="inlineStr">
+        <is>
+          <t>ASTREA: orçado R$ 112,07/mês, o que dá R$ 1.344,84 no ano — praticamente o valor de UMA das cinco parcelas (R$ 1.346,28). Quem montou a ficha tomou uma parcela pelo custo total do ano. O custo real da anuidade foi R$ 6.731,40, 5x o orçado. JUSBRASIL: orçado R$ 104,90/mês contra R$ 136,00 reais (1,3x), R$ 373,20 no ano. PAUTA PARA A REUNIÃO COM A DIRETORIA.</t>
+        </is>
+      </c>
+      <c r="D18" s="66" t="inlineStr">
+        <is>
+          <t>Subdimensionamento de R$ 5.759,76 no ano (R$ 5.386,56 do Astrea + R$ 373,20 do Jusbrasil). O planejado das duas linhas foi mantido como veio na ficha, de propósito, para o erro aparecer no comparativo em vez de ser corrigido em silêncio. Não é estouro de gestão: é erro na origem. Como o Astrea será cancelado, o efeito prático é só de 2026 — mas o método de orçar serviços parcelados precisa ser revisto para o ano que vem.</t>
+        </is>
+      </c>
+      <c r="E18" s="66" t="inlineStr">
+        <is>
+          <t>Cristiane + Diretoria</t>
+        </is>
+      </c>
+      <c r="F18" s="69" t="inlineStr">
+        <is>
+          <t>PAUTA REUNIÃO</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="58" customHeight="1">
+      <c r="A19" s="62" t="inlineStr">
+        <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B18" s="66" t="inlineStr">
+      <c r="B19" s="63" t="inlineStr">
         <is>
           <t>Competência x caixa — DECIDIR O REGIME</t>
         </is>
       </c>
-      <c r="C18" s="66" t="inlineStr">
+      <c r="C19" s="63" t="inlineStr">
         <is>
           <t>Confirmado pela gestora: TODOS os PJs das duas áreas prestam o serviço e recebem no mês seguinte — no Jurídico, Miguel, Thamar e Dra. Michele; no TI, Elias e Jonathan. O que foi pago em jan/26 é serviço de dez/2025, e o serviço de dez/26 só será pago em jan/2027. Hoje o realizado está lançado por CAIXA (mês do pagamento), que é como os valores foram informados, enquanto o orçamento foi montado por COMPETÊNCIA (mês do serviço). São bases diferentes no mesmo comparativo.</t>
         </is>
       </c>
-      <c r="D18" s="66" t="inlineStr">
+      <c r="D19" s="63" t="inlineStr">
         <is>
           <t>RECOMENDAÇÃO: migrar para competência, deslocando os PJs um mês para trás. Motivos: (1) o orçamento já é de competência, então acaba a comparação de bases diferentes; (2) por caixa, o ano de 2026 carrega um mês de 2025 e perde dez/26, o que distorce sempre que o valor muda no meio do ano — no Miguel, R$ 47.250 por caixa contra R$ 49.318 por competência em jan–jul, R$ 2.068 de diferença; (3) o SIENGE gera os dois regimes, então é escolha de configuração. Contra: caixa é mais fácil de bater com o extrato bancário. Decidir UMA vez e manter, senão o histórico mistura critérios. ATENÇÃO NO JONATHAN: o planejado dele começa em abr/26 (competência) e o realizado também foi lançado a partir de abr (caixa) — se ele recebe no mês seguinte, o pagamento de abril é serviço de março, e ou a entrada dele foi em março, ou o realizado de abril deveria ser zero. Conferir junto com a decisão do regime.</t>
         </is>
       </c>
-      <c r="E18" s="66" t="inlineStr">
+      <c r="E19" s="63" t="inlineStr">
         <is>
           <t>Cristiane + Financeiro</t>
         </is>
       </c>
-      <c r="F18" s="70" t="inlineStr">
+      <c r="F19" s="70" t="inlineStr">
         <is>
           <t>DECIDIR</t>
         </is>

</xml_diff>

<commit_message>
feat(orcamento): Elias renegociado, linha do AnyDesk e recomendacao de papelaria
Elias: R$ 1.065/mes ate ago e R$ 603,30 a partir de set/26, uma reducao
de 43% no valor mensal e R$ 1.846,80 no ano. Gestora confirmou que o
realizado de jan a jul e zero mesmo — contrato ativo sem acionamento —,
entao a economia de R$ 7.455 do periodo se mantem e a linha soma duas
economias de naturezas diferentes.

AnyDesk: linha criada com planejado zerado, a espera de valor e mes de
inicio. Registrada a sobreposicao a esclarecer com o J H Alves /
Monitor Remoto, que aparece no extrato com R$ 20.508,55 em sete meses e
tambem esta fora do orcamento — mesmo padrao do Jusfy x Astrea.

Orcamento do TI: R$ 284.971,50.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_JURIDICO_2026.xlsx
+++ b/orcamento/Orcamento_JURIDICO_2026.xlsx
@@ -16083,7 +16083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S32"/>
+  <dimension ref="A1:S33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -17017,49 +17017,49 @@
         <v/>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="43" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="43" t="inlineStr">
         <is>
           <t>TOTAL GERAL</t>
         </is>
       </c>
-      <c r="B32" s="43" t="n"/>
-      <c r="C32" s="43" t="n"/>
-      <c r="D32" s="43" t="n"/>
-      <c r="E32" s="43" t="n"/>
-      <c r="F32" s="44">
+      <c r="B33" s="43" t="n"/>
+      <c r="C33" s="43" t="n"/>
+      <c r="D33" s="43" t="n"/>
+      <c r="E33" s="43" t="n"/>
+      <c r="F33" s="44">
         <f>SUM(F6:F15)</f>
         <v/>
       </c>
-      <c r="G32" s="44">
+      <c r="G33" s="44">
         <f>SUM(G6:G15)</f>
         <v/>
       </c>
-      <c r="H32" s="44">
+      <c r="H33" s="44">
         <f>SUM(H6:H15)</f>
         <v/>
       </c>
-      <c r="I32" s="44">
+      <c r="I33" s="44">
         <f>SUM(I6:I15)</f>
         <v/>
       </c>
-      <c r="J32" s="44">
+      <c r="J33" s="44">
         <f>SUM(J6:J15)</f>
         <v/>
       </c>
-      <c r="K32" s="44">
+      <c r="K33" s="44">
         <f>SUM(K6:K15)</f>
         <v/>
       </c>
-      <c r="L32" s="45">
-        <f>IFERROR(K32/I32,"")</f>
-        <v/>
-      </c>
-      <c r="M32" s="45">
-        <f>IFERROR(J32/I32,"")</f>
-        <v/>
-      </c>
-      <c r="N32" s="43" t="n"/>
+      <c r="L33" s="45">
+        <f>IFERROR(K33/I33,"")</f>
+        <v/>
+      </c>
+      <c r="M33" s="45">
+        <f>IFERROR(J33/I33,"")</f>
+        <v/>
+      </c>
+      <c r="N33" s="43" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A5:N15"/>

</xml_diff>

<commit_message>
feat(orcamento): separa consultoria fixa do vinculo esporadico do mesmo prestador
Gestora esclareceu que "J H Alves - Monitor Remoto" tem dois vinculos
distintos: servicos esporadicos prestados de fora ate mar/26 e
consultoria fixa de 3 dias por semana desde abr/26.

TI-E03 passa a ser so a consultoria (planejado R$ 10.000/mes, realizado
R$ 16.196,99 em jan-jul, economia de R$ 53.803,01). Nova linha TI-E04
recebe o esporadico, com planejado zero e o unico pagamento de
R$ 4.311,56 em jan. A economia liquida do TI nao muda (R$ 56.946,45),
mas as duas historias deixam de se misturar numa linha so.

Papel do Vinicius atualizado no item Y: alem da rotina, ele faz suporte
ao usuario e apoio operacional ao desenvolvimento. Registrado o efeito
economico disso — cada tarefa operacional que sai do consultor por
R$ 31,25/h libera uma hora de R$ 60,58 das 104 mensais dele.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_JURIDICO_2026.xlsx
+++ b/orcamento/Orcamento_JURIDICO_2026.xlsx
@@ -16083,7 +16083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S33"/>
+  <dimension ref="A1:S34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -17017,49 +17017,49 @@
         <v/>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="43" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="43" t="inlineStr">
         <is>
           <t>TOTAL GERAL</t>
         </is>
       </c>
-      <c r="B33" s="43" t="n"/>
-      <c r="C33" s="43" t="n"/>
-      <c r="D33" s="43" t="n"/>
-      <c r="E33" s="43" t="n"/>
-      <c r="F33" s="44">
+      <c r="B34" s="43" t="n"/>
+      <c r="C34" s="43" t="n"/>
+      <c r="D34" s="43" t="n"/>
+      <c r="E34" s="43" t="n"/>
+      <c r="F34" s="44">
         <f>SUM(F6:F15)</f>
         <v/>
       </c>
-      <c r="G33" s="44">
+      <c r="G34" s="44">
         <f>SUM(G6:G15)</f>
         <v/>
       </c>
-      <c r="H33" s="44">
+      <c r="H34" s="44">
         <f>SUM(H6:H15)</f>
         <v/>
       </c>
-      <c r="I33" s="44">
+      <c r="I34" s="44">
         <f>SUM(I6:I15)</f>
         <v/>
       </c>
-      <c r="J33" s="44">
+      <c r="J34" s="44">
         <f>SUM(J6:J15)</f>
         <v/>
       </c>
-      <c r="K33" s="44">
+      <c r="K34" s="44">
         <f>SUM(K6:K15)</f>
         <v/>
       </c>
-      <c r="L33" s="45">
-        <f>IFERROR(K33/I33,"")</f>
-        <v/>
-      </c>
-      <c r="M33" s="45">
-        <f>IFERROR(J33/I33,"")</f>
-        <v/>
-      </c>
-      <c r="N33" s="43" t="n"/>
+      <c r="L34" s="45">
+        <f>IFERROR(K34/I34,"")</f>
+        <v/>
+      </c>
+      <c r="M34" s="45">
+        <f>IFERROR(J34/I34,"")</f>
+        <v/>
+      </c>
+      <c r="N34" s="43" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A5:N15"/>

</xml_diff>

<commit_message>
feat(orcamento): reclassificacao do Adapta solicitada ao financeiro
Decidido pedir a correcao agora, sem esperar a abertura do centro de
custo novo. Registrado o que pedir: reclassificar os seis lancamentos
do contrato 4134643529 (jan a jun/26) do centro de custo Juridico para
o de TI e ajustar a classificacao dos proximos, com conferencia quando
o centro de custo novo abrir.

Pendencia Q passa de RECLASSIFICAR para SOLICITADA.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_JURIDICO_2026.xlsx
+++ b/orcamento/Orcamento_JURIDICO_2026.xlsx
@@ -20282,7 +20282,7 @@
       </c>
       <c r="D16" s="66" t="inlineStr">
         <is>
-          <t>Reclassificar no SIENGE para o centro de custo correto e aplicar o rateio do item L. Enquanto não for corrigido, o Jurídico carrega R$ 3.351 que não são dele e o TI aparece sem um gasto que é seu — as duas áreas ficam com o comparativo errado. Aproveitar a abertura do novo centro de custo para acertar a classificação desde a origem.</t>
+          <t>DECIDIDO: solicitar a reclassificação contábil ao financeiro agora, sem esperar a abertura do centro de custo novo. Enquanto não for corrigido, o Jurídico carrega R$ 3.351 que não são dele e o TI aparece sem um gasto que é seu — as duas áreas ficam com o comparativo errado ao mesmo tempo. O que pedir ao financeiro: reclassificar os seis lançamentos do contrato 4134643529 (jan a jun/26) do centro de custo Jurídico para o de TI, e ajustar a classificação dos próximos para não repetir. Depois de reclassificado, aplicar o rateio do item L, já que é ferramenta de uso transversal. Quando o centro de custo novo abrir, conferir se a classificação nasceu certa.</t>
         </is>
       </c>
       <c r="E16" s="66" t="inlineStr">
@@ -20290,9 +20290,9 @@
           <t>Cristiane + Financeiro</t>
         </is>
       </c>
-      <c r="F16" s="64" t="inlineStr">
-        <is>
-          <t>RECLASSIFICAR</t>
+      <c r="F16" s="68" t="inlineStr">
+        <is>
+          <t>SOLICITADA</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(orcamento): CLT tambem deslocados para competencia
Gestora confirmou que Geovanna e Vinicius seguem a mesma regra dos PJs:
folha paga no mes seguinte ao da prestacao. Todo o realizado passa a
estar na mesma base, sem excecao.

O acumulado ate jun nao muda — o deslocamento apenas retira o mes de
jul, cujo servico so sera pago em agosto. A pendencia 7 deixa de ter a
duvida sobre os CLT; resta apenas confirmar se o aumento da Thamar
valeu para o servico de marco ou de abril.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_JURIDICO_2026.xlsx
+++ b/orcamento/Orcamento_JURIDICO_2026.xlsx
@@ -18328,9 +18328,7 @@
       <c r="M6" s="50" t="n">
         <v>2886.91</v>
       </c>
-      <c r="N6" s="50" t="n">
-        <v>2886.91</v>
-      </c>
+      <c r="N6" s="50" t="n"/>
       <c r="O6" s="50" t="n"/>
       <c r="P6" s="50" t="n"/>
       <c r="Q6" s="50" t="n"/>
@@ -18614,9 +18612,7 @@
       <c r="M10" s="50" t="n">
         <v>136</v>
       </c>
-      <c r="N10" s="50" t="n">
-        <v>136</v>
-      </c>
+      <c r="N10" s="50" t="n"/>
       <c r="O10" s="50" t="n"/>
       <c r="P10" s="50" t="n"/>
       <c r="Q10" s="50" t="n"/>
@@ -18764,9 +18760,7 @@
       <c r="M12" s="50" t="n">
         <v>970</v>
       </c>
-      <c r="N12" s="50" t="n">
-        <v>970</v>
-      </c>
+      <c r="N12" s="50" t="n"/>
       <c r="O12" s="50" t="n"/>
       <c r="P12" s="50" t="n"/>
       <c r="Q12" s="50" t="n"/>
@@ -18830,9 +18824,7 @@
       <c r="M13" s="50" t="n">
         <v>0</v>
       </c>
-      <c r="N13" s="50" t="n">
-        <v>0</v>
-      </c>
+      <c r="N13" s="50" t="n"/>
       <c r="O13" s="50" t="n"/>
       <c r="P13" s="50" t="n"/>
       <c r="Q13" s="50" t="n"/>
@@ -18900,9 +18892,7 @@
       <c r="M14" s="50" t="n">
         <v>0</v>
       </c>
-      <c r="N14" s="50" t="n">
-        <v>0</v>
-      </c>
+      <c r="N14" s="50" t="n"/>
       <c r="O14" s="50" t="n"/>
       <c r="P14" s="50" t="n"/>
       <c r="Q14" s="50" t="n"/>
@@ -20372,7 +20362,7 @@
       </c>
       <c r="D19" s="63" t="inlineStr">
         <is>
-          <t>Três efeitos. (1) O último mês completo passa a ser JUNHO, não julho: o serviço de jul só fecha quando sair o pagamento de ago — o mês de referência do Comparativo foi ajustado. (2) A conversão validou a entrada do Jonathan: por competência, o primeiro mês de serviço dele cai em abr, exatamente como informado. (3) O Monitor Remoto zerou no exercício — aquele pagamento de jan era serviço de dez/25. A CONFERIR: os CLT (Geovanna e Vinicius) NÃO foram deslocados. Se a folha for paga no mês seguinte, como é usual, eles também precisam deslocar. E na Thamar, confirmar se o aumento valeu para o serviço de mar ou de abr. Ao configurar a extração no SIENGE, travar o regime de competência e manter — trocar no meio do ano mistura critérios no histórico.</t>
+          <t>Três efeitos. (1) O último mês completo passa a ser JUNHO, não julho: o serviço de jul só fecha quando sair o pagamento de ago — o mês de referência do Comparativo foi ajustado. (2) A conversão validou a entrada do Jonathan: por competência, o primeiro mês de serviço dele cai em abr, exatamente como informado. (3) O Monitor Remoto zerou no exercício — aquele pagamento de jan era serviço de dez/25. Os CLT (Geovanna e Vinicius) seguem a mesma regra, confirmado pela gestora: folha paga no mês seguinte, também deslocados. A CONFERIR apenas na Thamar: se o aumento valeu para o serviço de mar ou de abr. Ao configurar a extração no SIENGE, travar o regime de competência e manter — trocar no meio do ano mistura critérios no histórico.</t>
         </is>
       </c>
       <c r="E19" s="63" t="inlineStr">

</xml_diff>